<commit_message>
BV-E9: ausführliche Excel-Vorlage neu erzeugt (Katalog v9)
Werkzeug Berichtsvorlage, Sammelbefehl alle, zweimal: zweiter Lauf
byte-gleich.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WuTkTgYBbZGmc25Uq4qwuU
</commit_message>
<xml_diff>
--- a/WindowsFormsApplication1/Allgemein/Bericht/Vorlagen/Berichtsvorlage_Excel_Ausfuehrlich.xlsx
+++ b/WindowsFormsApplication1/Allgemein/Bericht/Vorlagen/Berichtsvorlage_Excel_Ausfuehrlich.xlsx
@@ -7,14 +7,14 @@
   </x:bookViews>
   <x:sheets>
     <x:sheet name="Deckblatt" sheetId="1" r:id="rId2"/>
-    <x:sheet name="blatt.uebersicht" sheetId="2" r:id="rId3"/>
-    <x:sheet name="blatt.vergleich" sheetId="3" r:id="rId4"/>
-    <x:sheet name="Auswertung" sheetId="4" r:id="rId5"/>
-    <x:sheet name="Eigene Diagramme" sheetId="5" r:id="rId6"/>
-    <x:sheet name="blatt.wirtschaftlichkeit" sheetId="6" r:id="rId7"/>
-    <x:sheet name="blatt.verlauf" sheetId="7" r:id="rId8"/>
-    <x:sheet name="blatt.detail" sheetId="8" r:id="rId9"/>
-    <x:sheet name="blatt.checkliste" sheetId="9" r:id="rId10"/>
+    <x:sheet name="Projektübersicht" sheetId="2" r:id="rId3"/>
+    <x:sheet name="Variantenvergleich" sheetId="3" r:id="rId4"/>
+    <x:sheet name="blatt.wirtschaftlichkeit" sheetId="4" r:id="rId5"/>
+    <x:sheet name="Auswertung" sheetId="5" r:id="rId6"/>
+    <x:sheet name="Kapitalwertverlauf" sheetId="6" r:id="rId7"/>
+    <x:sheet name="blatt.detail" sheetId="7" r:id="rId8"/>
+    <x:sheet name="blatt.checkliste" sheetId="8" r:id="rId9"/>
+    <x:sheet name="Eigene Diagramme" sheetId="9" r:id="rId10"/>
     <x:sheet name="blatt.diagrammdaten" sheetId="10" r:id="rId11"/>
   </x:sheets>
   <x:definedNames>
@@ -48,6 +48,20 @@
         </x:r>
       </x:text>
     </x:comment>
+    <x:comment ref="A2" authorId="0">
+      <x:text>
+        <x:r>
+          <x:rPr>
+            <x:vertAlign val="baseline"/>
+            <x:sz val="9"/>
+            <x:color rgb="FF000000"/>
+            <x:rFont val="Tahoma"/>
+            <x:family val="2"/>
+          </x:rPr>
+          <x:t>Aufbau dieser Vorlage: Die Blätter „Projektübersicht“, „Variantenvergleich“, „Kapitalwertverlauf“ und das Musterblatt blatt.detail bilden die erzeugten Blätter Übersicht, Vergleich, Verlauf und Detail aus Einzelelementen nach — Zellplatzhalter, Tabellen und Diagramme, die Sie verschieben, löschen und umformatieren können. Die Eigenschaft EPOS.Blattanhang = nein (Datei › Informationen › Eigenschaften › Erweiterte Eigenschaften › Anpassen) sorgt dafür, dass EPOS die erzeugten Blätter ohne Blattmarke nicht zusätzlich anhängt. Formelmappe, Checkliste Anhang E und Diagrammdaten bleiben Blattmarken.</x:t>
+        </x:r>
+      </x:text>
+    </x:comment>
     <x:comment ref="A4" authorId="0">
       <x:text>
         <x:r>
@@ -292,7 +306,7 @@
             <x:rFont val="Tahoma"/>
             <x:family val="2"/>
           </x:rPr>
-          <x:t>Blattmarke der Diagrammdaten: die Zahlen aller Excel-Diagramme und der Reihennamen; am besten als letztes Blatt.</x:t>
+          <x:t>Blattmarke der Diagrammdaten: die Zahlen aller Excel-Diagramme und der Reihennamen; am besten als letztes Blatt. Das Blatt kommt auch ohne Marke hinzu, sobald die Mappe ein Diagramm trägt — die Diagramme zeigen auf seine Zahlen.</x:t>
         </x:r>
       </x:text>
     </x:comment>
@@ -316,7 +330,119 @@
             <x:rFont val="Tahoma"/>
             <x:family val="2"/>
           </x:rPr>
-          <x:t>Blattmarke allein in A1 eines leeren Blattes: An ihre Stelle tritt das erzeugte Blatt mit seinem gewohnten Namen; ohne Marke hängt es hinten an, ohne Inhalt entfällt es. Ein eigener Blattname gleich dem eines erzeugten Blattes wird umbenannt.</x:t>
+          <x:t>Nachbildung des Blattes „Übersicht“: Titel und Beschriftungen sind fester Text, die Werte Zellplatzhalter, darunter zwei Tabellen und ein Diagramm. Jedes Element lässt sich verschieben, löschen oder umformatieren; das erzeugte Blatt „Übersicht“ entsteht nicht zusätzlich.</x:t>
+        </x:r>
+      </x:text>
+    </x:comment>
+    <x:comment ref="B3" authorId="0">
+      <x:text>
+        <x:r>
+          <x:rPr>
+            <x:vertAlign val="baseline"/>
+            <x:sz val="9"/>
+            <x:color rgb="FF000000"/>
+            <x:rFont val="Tahoma"/>
+            <x:family val="2"/>
+          </x:rPr>
+          <x:t>Der Name des Stammprojekts. Zellplatzhalter: EPOS schreibt den Wert in diese Zelle. Beschriftung, Format und Lage der Zelle bestimmen Sie; ein anderer Schlüssel aus dem Katalog zeigt einen anderen Wert.</x:t>
+        </x:r>
+      </x:text>
+    </x:comment>
+    <x:comment ref="B4" authorId="0">
+      <x:text>
+        <x:r>
+          <x:rPr>
+            <x:vertAlign val="baseline"/>
+            <x:sz val="9"/>
+            <x:color rgb="FF000000"/>
+            <x:rFont val="Tahoma"/>
+            <x:family val="2"/>
+          </x:rPr>
+          <x:t>Der Kunde des Stammprojekts; leer, wenn keiner eingetragen ist. Zellplatzhalter: EPOS schreibt den Wert in diese Zelle. Beschriftung, Format und Lage der Zelle bestimmen Sie; ein anderer Schlüssel aus dem Katalog zeigt einen anderen Wert.</x:t>
+        </x:r>
+      </x:text>
+    </x:comment>
+    <x:comment ref="B5" authorId="0">
+      <x:text>
+        <x:r>
+          <x:rPr>
+            <x:vertAlign val="baseline"/>
+            <x:sz val="9"/>
+            <x:color rgb="FF000000"/>
+            <x:rFont val="Tahoma"/>
+            <x:family val="2"/>
+          </x:rPr>
+          <x:t>Die Person, die das Stammprojekt bearbeitet; leer, wenn keine eingetragen ist. Zellplatzhalter: EPOS schreibt den Wert in diese Zelle. Beschriftung, Format und Lage der Zelle bestimmen Sie; ein anderer Schlüssel aus dem Katalog zeigt einen anderen Wert.</x:t>
+        </x:r>
+      </x:text>
+    </x:comment>
+    <x:comment ref="B6" authorId="0">
+      <x:text>
+        <x:r>
+          <x:rPr>
+            <x:vertAlign val="baseline"/>
+            <x:sz val="9"/>
+            <x:color rgb="FF000000"/>
+            <x:rFont val="Tahoma"/>
+            <x:family val="2"/>
+          </x:rPr>
+          <x:t>Die Klimaregion des Stammprojekts. Zellplatzhalter: EPOS schreibt den Wert in diese Zelle. Beschriftung, Format und Lage der Zelle bestimmen Sie; ein anderer Schlüssel aus dem Katalog zeigt einen anderen Wert.</x:t>
+        </x:r>
+      </x:text>
+    </x:comment>
+    <x:comment ref="B7" authorId="0">
+      <x:text>
+        <x:r>
+          <x:rPr>
+            <x:vertAlign val="baseline"/>
+            <x:sz val="9"/>
+            <x:color rgb="FF000000"/>
+            <x:rFont val="Tahoma"/>
+            <x:family val="2"/>
+          </x:rPr>
+          <x:t>Erstellungsdatum des Berichts, nach der Sprache des Berichts formatiert; in Excel ein echtes Datum. Datum mit Uhrzeit (Formatangabe |datum mit zeit): ein echter Excel-Datumswert; ohne die Angabe das kurze Datum.</x:t>
+        </x:r>
+      </x:text>
+    </x:comment>
+    <x:comment ref="A9" authorId="0">
+      <x:text>
+        <x:r>
+          <x:rPr>
+            <x:vertAlign val="baseline"/>
+            <x:sz val="9"/>
+            <x:color rgb="FF000000"/>
+            <x:rFont val="Tahoma"/>
+            <x:family val="2"/>
+          </x:rPr>
+          <x:t>Tabelle der Stände: Rolle, Bezeichner, Projektname, Simulation vom, Hinweis und Stromspeicher. Tabelle als Zellmarke: EPOS schreibt sie ab dieser Zelle und fügt dafür Zeilen ein; Inhalte darunter wandern mit, die Spalten rechts müssen frei sein. Diese Tabelle ist listentauglich und wird zugleich eine Excel-Tabelle EPOS_tabelle__varianten.</x:t>
+        </x:r>
+      </x:text>
+    </x:comment>
+    <x:comment ref="A11" authorId="0">
+      <x:text>
+        <x:r>
+          <x:rPr>
+            <x:vertAlign val="baseline"/>
+            <x:sz val="9"/>
+            <x:color rgb="FF000000"/>
+            <x:rFont val="Tahoma"/>
+            <x:family val="2"/>
+          </x:rPr>
+          <x:t>Tabelle Gewerk × Stand: welche Komponenten jeder Stand führt (✓, ✓ (Anzahl) oder —); Spalten je Stand in Blöcken zu drei Varianten. Tabelle mit Spalten je Stand oder Gruppenzeilen: ein formatierter Bereich ohne Excel-Tabelle.</x:t>
+        </x:r>
+      </x:text>
+    </x:comment>
+    <x:comment ref="A13" authorId="0">
+      <x:text>
+        <x:r>
+          <x:rPr>
+            <x:vertAlign val="baseline"/>
+            <x:sz val="9"/>
+            <x:color rgb="FF000000"/>
+            <x:rFont val="Tahoma"/>
+            <x:family val="2"/>
+          </x:rPr>
+          <x:t>Bild des Stammprojekts: Speichertemperaturen (oberste und unterste Schicht) in drei Wochen — braucht die Stundenreihen des Laufs. Bildplatzhalter: Hier entsteht ein Excel-Diagramm (zehn Spalten × zwanzig Zeilen) mit den Zahlen des Blattes „Diagrammdaten“. Verschieben oder löschen Sie die Zelle; das fertige Diagramm formatieren Sie in Excel.</x:t>
         </x:r>
       </x:text>
     </x:comment>
@@ -340,7 +466,63 @@
             <x:rFont val="Tahoma"/>
             <x:family val="2"/>
           </x:rPr>
-          <x:t>Blattmarke allein in A1 eines leeren Blattes: An ihre Stelle tritt das erzeugte Blatt mit seinem gewohnten Namen; ohne Marke hängt es hinten an, ohne Inhalt entfällt es. Ein eigener Blattname gleich dem eines erzeugten Blattes wird umbenannt.</x:t>
+          <x:t>Nur Excel: die Vergleichsliste des Blattes „Vergleich“ — je Kennzahl eine Zeile mit Gruppe und Einheit, je Stand eine Spalte, rechts Δ % je Variante gegen den Stamm; ohne Gruppenzeilen, auch als Excel-Tabelle EPOS_tabelle__vergleich__liste. Nachbildung des Blattes „Vergleich“: die Vergleichsliste tabelle.vergleich.liste — je Kennzahl eine Zeile mit Gruppe und Einheit, je Stand eine Spalte, rechts Δ % je Variante; eine Excel-Tabelle EPOS_tabelle__vergleich__liste mit Filter. Die Δ-Werte stehen als Zahlen, im erzeugten Blatt als Formeln. Andere Tafeln des Vergleichs: tabelle.vergleich mit Gruppenzeilen, tabelle.vergleich.&lt;gruppe&gt; je Gruppe.</x:t>
+        </x:r>
+      </x:text>
+    </x:comment>
+    <x:comment ref="A3" authorId="0">
+      <x:text>
+        <x:r>
+          <x:rPr>
+            <x:vertAlign val="baseline"/>
+            <x:sz val="9"/>
+            <x:color rgb="FF000000"/>
+            <x:rFont val="Tahoma"/>
+            <x:family val="2"/>
+          </x:rPr>
+          <x:t>Bild: Brennstoffeinsatz gesamt je Stand als Balken (Stamm hervorgehoben); ab zwei Ständen mit Wert. Bildplatzhalter: Hier entsteht ein Excel-Diagramm (zehn Spalten × zwanzig Zeilen) mit den Zahlen des Blattes „Diagrammdaten“. Verschieben oder löschen Sie die Zelle; das fertige Diagramm formatieren Sie in Excel. Vergleichsbalken einer Kennzahl (bild.vergleich.balken.&lt;kennzahl&gt;) als Excel-Diagramm — erst ab zwei Ständen; mit einem Stand bleibt die Zelle leer. Die vier Balken des erzeugten Blattes stehen untereinander; löschen Sie, was Sie nicht brauchen.</x:t>
+        </x:r>
+      </x:text>
+    </x:comment>
+    <x:comment ref="A25" authorId="0">
+      <x:text>
+        <x:r>
+          <x:rPr>
+            <x:vertAlign val="baseline"/>
+            <x:sz val="9"/>
+            <x:color rgb="FF000000"/>
+            <x:rFont val="Tahoma"/>
+            <x:family val="2"/>
+          </x:rPr>
+          <x:t>Bild: Netzbezug Strom je Stand als Balken (Stamm hervorgehoben); ab zwei Ständen mit Wert. Bildplatzhalter: Hier entsteht ein Excel-Diagramm (zehn Spalten × zwanzig Zeilen) mit den Zahlen des Blattes „Diagrammdaten“. Verschieben oder löschen Sie die Zelle; das fertige Diagramm formatieren Sie in Excel.</x:t>
+        </x:r>
+      </x:text>
+    </x:comment>
+    <x:comment ref="A47" authorId="0">
+      <x:text>
+        <x:r>
+          <x:rPr>
+            <x:vertAlign val="baseline"/>
+            <x:sz val="9"/>
+            <x:color rgb="FF000000"/>
+            <x:rFont val="Tahoma"/>
+            <x:family val="2"/>
+          </x:rPr>
+          <x:t>Bild: Wärmerestbedarf (ungedeckt) je Stand als Balken (Stamm hervorgehoben); ab zwei Ständen mit Wert. Bildplatzhalter: Hier entsteht ein Excel-Diagramm (zehn Spalten × zwanzig Zeilen) mit den Zahlen des Blattes „Diagrammdaten“. Verschieben oder löschen Sie die Zelle; das fertige Diagramm formatieren Sie in Excel.</x:t>
+        </x:r>
+      </x:text>
+    </x:comment>
+    <x:comment ref="A69" authorId="0">
+      <x:text>
+        <x:r>
+          <x:rPr>
+            <x:vertAlign val="baseline"/>
+            <x:sz val="9"/>
+            <x:color rgb="FF000000"/>
+            <x:rFont val="Tahoma"/>
+            <x:family val="2"/>
+          </x:rPr>
+          <x:t>Bild: Jahresarbeitszahl (JAZ) WP je Stand als Balken (Stamm hervorgehoben); ab zwei Ständen mit Wert. Bildplatzhalter: Hier entsteht ein Excel-Diagramm (zehn Spalten × zwanzig Zeilen) mit den Zahlen des Blattes „Diagrammdaten“. Verschieben oder löschen Sie die Zelle; das fertige Diagramm formatieren Sie in Excel.</x:t>
         </x:r>
       </x:text>
     </x:comment>
@@ -354,73 +536,17 @@
     <x:author>EPOS-Plan</x:author>
   </x:authors>
   <x:commentList>
-    <x:comment ref="A4" authorId="0">
-      <x:text>
-        <x:r>
-          <x:rPr>
-            <x:vertAlign val="baseline"/>
-            <x:sz val="9"/>
-            <x:color rgb="FF000000"/>
-            <x:rFont val="Tahoma"/>
-            <x:family val="2"/>
-          </x:rPr>
-          <x:t>Tabelle als Zellmarke: EPOS schreibt sie ab dieser Zelle und fügt dafür Zeilen ein; Inhalte darunter wandern mit, die Spalten rechts müssen frei sein. Diese Tabelle ist listentauglich und wird zugleich eine Excel-Tabelle EPOS_tabelle__varianten.</x:t>
-        </x:r>
-      </x:text>
-    </x:comment>
-    <x:comment ref="A7" authorId="0">
-      <x:text>
-        <x:r>
-          <x:rPr>
-            <x:vertAlign val="baseline"/>
-            <x:sz val="9"/>
-            <x:color rgb="FF000000"/>
-            <x:rFont val="Tahoma"/>
-            <x:family val="2"/>
-          </x:rPr>
-          <x:t>Tabelle mit Spalten je Stand oder Gruppenzeilen: ein formatierter Bereich ohne Excel-Tabelle.</x:t>
-        </x:r>
-      </x:text>
-    </x:comment>
-    <x:comment ref="A10" authorId="0">
-      <x:text>
-        <x:r>
-          <x:rPr>
-            <x:vertAlign val="baseline"/>
-            <x:sz val="9"/>
-            <x:color rgb="FF000000"/>
-            <x:rFont val="Tahoma"/>
-            <x:family val="2"/>
-          </x:rPr>
-          <x:t>Tabelle mit reiner Excel-Quelle (Parameterblock, Kapitalwertverlauf): dieselben Zahlen wie in den erzeugten Blättern, hier an einer Stelle Ihrer Wahl.</x:t>
-        </x:r>
-      </x:text>
-    </x:comment>
-    <x:comment ref="A13" authorId="0">
-      <x:text>
-        <x:r>
-          <x:rPr>
-            <x:vertAlign val="baseline"/>
-            <x:sz val="9"/>
-            <x:color rgb="FF000000"/>
-            <x:rFont val="Tahoma"/>
-            <x:family val="2"/>
-          </x:rPr>
-          <x:t>Tabelle mit reiner Excel-Quelle (Parameterblock, Kapitalwertverlauf): dieselben Zahlen wie in den erzeugten Blättern, hier an einer Stelle Ihrer Wahl.</x:t>
-        </x:r>
-      </x:text>
-    </x:comment>
-    <x:comment ref="A16" authorId="0">
-      <x:text>
-        <x:r>
-          <x:rPr>
-            <x:vertAlign val="baseline"/>
-            <x:sz val="9"/>
-            <x:color rgb="FF000000"/>
-            <x:rFont val="Tahoma"/>
-            <x:family val="2"/>
-          </x:rPr>
-          <x:t>Bildplatzhalter allein in einer Zelle: Hier entsteht ein Excel-Diagramm mit Daten (zehn Spalten × zwanzig Zeilen) — dieselben Zahlen wie im Bild des Wortberichts.</x:t>
+    <x:comment ref="A1" authorId="0">
+      <x:text>
+        <x:r>
+          <x:rPr>
+            <x:vertAlign val="baseline"/>
+            <x:sz val="9"/>
+            <x:color rgb="FF000000"/>
+            <x:rFont val="Tahoma"/>
+            <x:family val="2"/>
+          </x:rPr>
+          <x:t>Blattmarke der Formelmappe (Blatt „Wirtschaftlichkeit“) samt ihren Diagrammen. Sie bleibt eine Blattmarke: Ihre Zellen tragen lebende Formeln auf die reservierten Namen (Zins_i, Zeitraum_T …) und eine Gegenrechnung, deren Lage von den Daten abhängt — aus Einzelelementen lässt sie sich nicht nachbauen. Dieselben Zahlen ohne Formeln stehen als Einzelelemente auf dem Blatt „Auswertung“ und auf dem Musterblatt; brauchen Sie nur eines, löschen Sie das andere.</x:t>
         </x:r>
       </x:text>
     </x:comment>
@@ -444,21 +570,189 @@
             <x:rFont val="Tahoma"/>
             <x:family val="2"/>
           </x:rPr>
-          <x:t>Excel-Tabelle mit dem Namen EPOS_tabelle__wirtschaft__szenarien: EPOS füllt sie Zeile für Zeile, sie wächst oder schrumpft. Das Säulendiagramm rechts zeigt auf ihre Datenzeilen — EPOS zieht seine Bezüge mit und trägt die neuen Werte ein.</x:t>
-        </x:r>
-      </x:text>
-    </x:comment>
-    <x:comment ref="A29" authorId="0">
-      <x:text>
-        <x:r>
-          <x:rPr>
-            <x:vertAlign val="baseline"/>
-            <x:sz val="9"/>
-            <x:color rgb="FF000000"/>
-            <x:rFont val="Tahoma"/>
-            <x:family val="2"/>
-          </x:rPr>
-          <x:t>Die Namen EPOS.reihe.monate und EPOS.reihe.waermebedarf.monate zeigen hier auf zwölf Zellen; das Liniendiagramm rechts nutzt die Namen. Beim Füllen setzt EPOS die Namen auf die Monatssummen des Stammprojekts im Blatt „Diagrammdaten“.</x:t>
+          <x:t>Die Wirtschaftlichkeit in Einzelelementen: Parameter, Kennzahlen je Szenario, Bandbreite, Vorschlag, nicht monetarisierbare Wirkungen, Hinweise und die vier Diagramme der Formelmappe — dieselben Zahlen als Werte, frei anzuordnen. Die Tafeln je Stand (Betriebskosten, KWK-Zuschlag, Mehrjahrestabelle, Zahlungsstrom) stehen auf dem Musterblatt.</x:t>
+        </x:r>
+      </x:text>
+    </x:comment>
+    <x:comment ref="A4" authorId="0">
+      <x:text>
+        <x:r>
+          <x:rPr>
+            <x:vertAlign val="baseline"/>
+            <x:sz val="9"/>
+            <x:color rgb="FF000000"/>
+            <x:rFont val="Tahoma"/>
+            <x:family val="2"/>
+          </x:rPr>
+          <x:t>Nur Excel: der Parameterblock der Formelmappe — Kalkulationszins, Betrachtungszeitraum, Preissteigerungen und die Änderungen der Szenarien Erwartet, Günstig und Ungünstig als Anteil, die Namen der Formelmappe und die gepflegten Trägerpreise. Tabelle mit reiner Excel-Quelle (Parameterblock, Kapitalwertverlauf): dieselben Zahlen wie in den erzeugten Blättern, hier an einer Stelle Ihrer Wahl.</x:t>
+        </x:r>
+      </x:text>
+    </x:comment>
+    <x:comment ref="A7" authorId="0">
+      <x:text>
+        <x:r>
+          <x:rPr>
+            <x:vertAlign val="baseline"/>
+            <x:sz val="9"/>
+            <x:color rgb="FF000000"/>
+            <x:rFont val="Tahoma"/>
+            <x:family val="2"/>
+          </x:rPr>
+          <x:t>Kennzahltafel der Wirtschaftlichkeit im Szenario „Erwartet“: je Stand eine Spalte, in der Paarsicht A | B. Tabelle als Zellmarke: EPOS schreibt sie ab dieser Zelle und fügt dafür Zeilen ein, Inhalte darunter wandern mit. Verschieben Sie die Zelle, um die Tabelle zu verschieben; löschen Sie sie, um die Tabelle wegzulassen.</x:t>
+        </x:r>
+      </x:text>
+    </x:comment>
+    <x:comment ref="A10" authorId="0">
+      <x:text>
+        <x:r>
+          <x:rPr>
+            <x:vertAlign val="baseline"/>
+            <x:sz val="9"/>
+            <x:color rgb="FF000000"/>
+            <x:rFont val="Tahoma"/>
+            <x:family val="2"/>
+          </x:rPr>
+          <x:t>Kennzahltafel der Wirtschaftlichkeit im Szenario „Günstig“: je Stand eine Spalte, in der Paarsicht A | B. Tabelle als Zellmarke: EPOS schreibt sie ab dieser Zelle und fügt dafür Zeilen ein, Inhalte darunter wandern mit. Verschieben Sie die Zelle, um die Tabelle zu verschieben; löschen Sie sie, um die Tabelle wegzulassen.</x:t>
+        </x:r>
+      </x:text>
+    </x:comment>
+    <x:comment ref="A13" authorId="0">
+      <x:text>
+        <x:r>
+          <x:rPr>
+            <x:vertAlign val="baseline"/>
+            <x:sz val="9"/>
+            <x:color rgb="FF000000"/>
+            <x:rFont val="Tahoma"/>
+            <x:family val="2"/>
+          </x:rPr>
+          <x:t>Kennzahltafel der Wirtschaftlichkeit im Szenario „Ungünstig“: je Stand eine Spalte, in der Paarsicht A | B. Tabelle als Zellmarke: EPOS schreibt sie ab dieser Zelle und fügt dafür Zeilen ein, Inhalte darunter wandern mit. Verschieben Sie die Zelle, um die Tabelle zu verschieben; löschen Sie sie, um die Tabelle wegzulassen.</x:t>
+        </x:r>
+      </x:text>
+    </x:comment>
+    <x:comment ref="A16" authorId="0">
+      <x:text>
+        <x:r>
+          <x:rPr>
+            <x:vertAlign val="baseline"/>
+            <x:sz val="9"/>
+            <x:color rgb="FF000000"/>
+            <x:rFont val="Tahoma"/>
+            <x:family val="2"/>
+          </x:rPr>
+          <x:t>Szenarienübersicht: Referenzzeile und je Version ΔKW in Ungünstig, Erwartet und Günstig, Spanne, Amortisation und Einstufung. Tabelle als Zellmarke: EPOS schreibt sie ab dieser Zelle und fügt dafür Zeilen ein, Inhalte darunter wandern mit. Verschieben Sie die Zelle, um die Tabelle zu verschieben; löschen Sie sie, um die Tabelle wegzulassen.</x:t>
+        </x:r>
+      </x:text>
+    </x:comment>
+    <x:comment ref="A19" authorId="0">
+      <x:text>
+        <x:r>
+          <x:rPr>
+            <x:vertAlign val="baseline"/>
+            <x:sz val="9"/>
+            <x:color rgb="FF000000"/>
+            <x:rFont val="Tahoma"/>
+            <x:family val="2"/>
+          </x:rPr>
+          <x:t>Vorschlag zur Entscheidung aus der Bewertung; entfällt, wenn leer. Zellplatzhalter: EPOS schreibt den Wert in diese Zelle. Beschriftung, Format und Lage der Zelle bestimmen Sie; ein anderer Schlüssel aus dem Katalog zeigt einen anderen Wert.</x:t>
+        </x:r>
+      </x:text>
+    </x:comment>
+    <x:comment ref="A22" authorId="0">
+      <x:text>
+        <x:r>
+          <x:rPr>
+            <x:vertAlign val="baseline"/>
+            <x:sz val="9"/>
+            <x:color rgb="FF000000"/>
+            <x:rFont val="Tahoma"/>
+            <x:family val="2"/>
+          </x:rPr>
+          <x:t>Tabelle der nicht monetarisierbaren Wirkungen: Kategorie, Beschreibung, Dauer, Wirkung auf Organisation, Mitarbeiter und Umwelt, Beurteilung. Tabelle als Zellmarke: EPOS schreibt sie ab dieser Zelle und fügt dafür Zeilen ein, Inhalte darunter wandern mit. Verschieben Sie die Zelle, um die Tabelle zu verschieben; löschen Sie sie, um die Tabelle wegzulassen.</x:t>
+        </x:r>
+      </x:text>
+    </x:comment>
+    <x:comment ref="A25" authorId="0">
+      <x:text>
+        <x:r>
+          <x:rPr>
+            <x:vertAlign val="baseline"/>
+            <x:sz val="9"/>
+            <x:color rgb="FF000000"/>
+            <x:rFont val="Tahoma"/>
+            <x:family val="2"/>
+          </x:rPr>
+          <x:t>Hinweise der Rechnung je Stand („⚠ Stand: Hinweis“) im Szenario „Erwartet“. Zellplatzhalter: EPOS schreibt den Wert in diese Zelle. Beschriftung, Format und Lage der Zelle bestimmen Sie; ein anderer Schlüssel aus dem Katalog zeigt einen anderen Wert.</x:t>
+        </x:r>
+      </x:text>
+    </x:comment>
+    <x:comment ref="A26" authorId="0">
+      <x:text>
+        <x:r>
+          <x:rPr>
+            <x:vertAlign val="baseline"/>
+            <x:sz val="9"/>
+            <x:color rgb="FF000000"/>
+            <x:rFont val="Tahoma"/>
+            <x:family val="2"/>
+          </x:rPr>
+          <x:t>Gültigkeitshinweise der Wirtschaftlichkeit über alle Stände: keine Rechnung, Rückfall auf den gespeicherten Stand, veraltete Ergebnisse, Fehlgründe, Warnungen der Kennzahltafel. Zellplatzhalter: EPOS schreibt den Wert in diese Zelle. Beschriftung, Format und Lage der Zelle bestimmen Sie; ein anderer Schlüssel aus dem Katalog zeigt einen anderen Wert.</x:t>
+        </x:r>
+      </x:text>
+    </x:comment>
+    <x:comment ref="A28" authorId="0">
+      <x:text>
+        <x:r>
+          <x:rPr>
+            <x:vertAlign val="baseline"/>
+            <x:sz val="9"/>
+            <x:color rgb="FF000000"/>
+            <x:rFont val="Tahoma"/>
+            <x:family val="2"/>
+          </x:rPr>
+          <x:t>Bild: kumulierter Barwert der Differenz zur Referenz in allen drei Szenarien. Bildplatzhalter: Hier entsteht ein Excel-Diagramm (zehn Spalten × zwanzig Zeilen) mit den Zahlen des Blattes „Diagrammdaten“. Verschieben oder löschen Sie die Zelle; das fertige Diagramm formatieren Sie in Excel.</x:t>
+        </x:r>
+      </x:text>
+    </x:comment>
+    <x:comment ref="A50" authorId="0">
+      <x:text>
+        <x:r>
+          <x:rPr>
+            <x:vertAlign val="baseline"/>
+            <x:sz val="9"/>
+            <x:color rgb="FF000000"/>
+            <x:rFont val="Tahoma"/>
+            <x:family val="2"/>
+          </x:rPr>
+          <x:t>Bild: kumulierte Barwerte je Version im Szenario „Erwartet“. Bildplatzhalter: Hier entsteht ein Excel-Diagramm (zehn Spalten × zwanzig Zeilen) mit den Zahlen des Blattes „Diagrammdaten“. Verschieben oder löschen Sie die Zelle; das fertige Diagramm formatieren Sie in Excel.</x:t>
+        </x:r>
+      </x:text>
+    </x:comment>
+    <x:comment ref="A72" authorId="0">
+      <x:text>
+        <x:r>
+          <x:rPr>
+            <x:vertAlign val="baseline"/>
+            <x:sz val="9"/>
+            <x:color rgb="FF000000"/>
+            <x:rFont val="Tahoma"/>
+            <x:family val="2"/>
+          </x:rPr>
+          <x:t>Bild: von der Investition zur Kapitalwertdifferenz der Leitversion (Brücke) — nur, wenn sie nicht die Referenz ist. Bildplatzhalter: Hier entsteht ein Excel-Diagramm (zehn Spalten × zwanzig Zeilen) mit den Zahlen des Blattes „Diagrammdaten“. Verschieben oder löschen Sie die Zelle; das fertige Diagramm formatieren Sie in Excel.</x:t>
+        </x:r>
+      </x:text>
+    </x:comment>
+    <x:comment ref="A94" authorId="0">
+      <x:text>
+        <x:r>
+          <x:rPr>
+            <x:vertAlign val="baseline"/>
+            <x:sz val="9"/>
+            <x:color rgb="FF000000"/>
+            <x:rFont val="Tahoma"/>
+            <x:family val="2"/>
+          </x:rPr>
+          <x:t>Bild: Spanne der Kapitalwertdifferenz je Version über die drei Szenarien. Bildplatzhalter: Hier entsteht ein Excel-Diagramm (zehn Spalten × zwanzig Zeilen) mit den Zahlen des Blattes „Diagrammdaten“. Verschieben oder löschen Sie die Zelle; das fertige Diagramm formatieren Sie in Excel.</x:t>
         </x:r>
       </x:text>
     </x:comment>
@@ -472,17 +766,17 @@
     <x:author>EPOS-Plan</x:author>
   </x:authors>
   <x:commentList>
-    <x:comment ref="A1" authorId="0">
-      <x:text>
-        <x:r>
-          <x:rPr>
-            <x:vertAlign val="baseline"/>
-            <x:sz val="9"/>
-            <x:color rgb="FF000000"/>
-            <x:rFont val="Tahoma"/>
-            <x:family val="2"/>
-          </x:rPr>
-          <x:t>Blattmarke der Formelmappe (Blatt „Wirtschaftlichkeit“): Parameterblock mit den reservierten Namen, Mehrjahrestabellen und Kennzahlen in Formeln, dazu ihre Diagramme.</x:t>
+    <x:comment ref="A3" authorId="0">
+      <x:text>
+        <x:r>
+          <x:rPr>
+            <x:vertAlign val="baseline"/>
+            <x:sz val="9"/>
+            <x:color rgb="FF000000"/>
+            <x:rFont val="Tahoma"/>
+            <x:family val="2"/>
+          </x:rPr>
+          <x:t>Nur Excel: der Kapitalwertverlauf je Jahr — je Szenario und Stand eine Spalte, darunter Nulldurchgang, Restwert und Kapitalwertdifferenz (wie das Blatt „Verlauf“); verbundene Köpfe, ein erzeugter Bereich. Nachbildung des Blattes „Verlauf“: der Kapitalwertverlauf je Jahr als erzeugter Bereich (tabelle.wirtschaft.verlauf), darunter die Statuszeile. Ohne Verlauf bleibt die Zelle leer — anders als im erzeugten Bericht entfällt das Blatt nicht; löschen Sie es, wenn Sie es nie brauchen.</x:t>
         </x:r>
       </x:text>
     </x:comment>
@@ -506,7 +800,259 @@
             <x:rFont val="Tahoma"/>
             <x:family val="2"/>
           </x:rPr>
-          <x:t>Blattmarke allein in A1 eines leeren Blattes: An ihre Stelle tritt das erzeugte Blatt mit seinem gewohnten Namen; ohne Marke hängt es hinten an, ohne Inhalt entfällt es. Ein eigener Blattname gleich dem eines erzeugten Blattes wird umbenannt.</x:t>
+          <x:t>Musterblatt: Die Blattmarke blatt.detail auf einem Blatt mit weiteren Zellen — EPOS legt je Stand eine Kopie an, benannt wie das Detailblatt, und füllt ihre Platzhalter stand.* mit den Werten dieses Stands. Es bildet das Detailblatt nach (Kopf, Kennzahlen, Erzeuger, Brennstoffmengen, Monatswerte, vier Diagramme), dazu je Stand die Deckungskreise des Vergleichs und die Tafeln der Wirtschaftlichkeit.</x:t>
+        </x:r>
+      </x:text>
+    </x:comment>
+    <x:comment ref="A2" authorId="0">
+      <x:text>
+        <x:r>
+          <x:rPr>
+            <x:vertAlign val="baseline"/>
+            <x:sz val="9"/>
+            <x:color rgb="FF000000"/>
+            <x:rFont val="Tahoma"/>
+            <x:family val="2"/>
+          </x:rPr>
+          <x:t>Werte je Stand (stand.*) stehen nur auf dem Musterblatt; Excel kennt keine Blöcke wie Word.</x:t>
+        </x:r>
+      </x:text>
+    </x:comment>
+    <x:comment ref="B3" authorId="0">
+      <x:text>
+        <x:r>
+          <x:rPr>
+            <x:vertAlign val="baseline"/>
+            <x:sz val="9"/>
+            <x:color rgb="FF000000"/>
+            <x:rFont val="Tahoma"/>
+            <x:family val="2"/>
+          </x:rPr>
+          <x:t>Datum und Uhrzeit des Simulationslaufs des laufenden Stands. Zellplatzhalter: EPOS schreibt den Wert in diese Zelle. Beschriftung, Format und Lage der Zelle bestimmen Sie; ein anderer Schlüssel aus dem Katalog zeigt einen anderen Wert.</x:t>
+        </x:r>
+      </x:text>
+    </x:comment>
+    <x:comment ref="A4" authorId="0">
+      <x:text>
+        <x:r>
+          <x:rPr>
+            <x:vertAlign val="baseline"/>
+            <x:sz val="9"/>
+            <x:color rgb="FF000000"/>
+            <x:rFont val="Tahoma"/>
+            <x:family val="2"/>
+          </x:rPr>
+          <x:t>Fehlertext des laufenden Stands; leer ohne Fehler. Zellplatzhalter: EPOS schreibt den Wert in diese Zelle. Beschriftung, Format und Lage der Zelle bestimmen Sie; ein anderer Schlüssel aus dem Katalog zeigt einen anderen Wert.</x:t>
+        </x:r>
+      </x:text>
+    </x:comment>
+    <x:comment ref="A6" authorId="0">
+      <x:text>
+        <x:r>
+          <x:rPr>
+            <x:vertAlign val="baseline"/>
+            <x:sz val="9"/>
+            <x:color rgb="FF000000"/>
+            <x:rFont val="Tahoma"/>
+            <x:family val="2"/>
+          </x:rPr>
+          <x:t>Nur Excel: alle Kennzahlen des Stands wie im Detailblatt — Gruppe, Kennzahl, Wert und Einheit je Kennzahl mit Wert; auf dem Musterblatt als Zellmarke, zugleich Excel-Tabelle. Tabelle je Stand als Zellmarke auf dem Musterblatt: je Kopie die Tabelle ihres Stands.</x:t>
+        </x:r>
+      </x:text>
+    </x:comment>
+    <x:comment ref="A9" authorId="0">
+      <x:text>
+        <x:r>
+          <x:rPr>
+            <x:vertAlign val="baseline"/>
+            <x:sz val="9"/>
+            <x:color rgb="FF000000"/>
+            <x:rFont val="Tahoma"/>
+            <x:family val="2"/>
+          </x:rPr>
+          <x:t>Die Erzeuger des laufenden Stands je Gerät: Wärme, Strom, Energieträger und Verbrauch; nur im Block #je stand. Tabelle je Stand als Zellmarke auf dem Musterblatt: je Kopie die Tabelle ihres Stands.</x:t>
+        </x:r>
+      </x:text>
+    </x:comment>
+    <x:comment ref="A12" authorId="0">
+      <x:text>
+        <x:r>
+          <x:rPr>
+            <x:vertAlign val="baseline"/>
+            <x:sz val="9"/>
+            <x:color rgb="FF000000"/>
+            <x:rFont val="Tahoma"/>
+            <x:family val="2"/>
+          </x:rPr>
+          <x:t>Die Brennstoffmengen des laufenden Stands in der Abrechnungseinheit; nur im Block #je stand. Tabelle je Stand als Zellmarke auf dem Musterblatt: je Kopie die Tabelle ihres Stands.</x:t>
+        </x:r>
+      </x:text>
+    </x:comment>
+    <x:comment ref="A14" authorId="0">
+      <x:text>
+        <x:r>
+          <x:rPr>
+            <x:vertAlign val="baseline"/>
+            <x:sz val="9"/>
+            <x:color rgb="FF000000"/>
+            <x:rFont val="Tahoma"/>
+            <x:family val="2"/>
+          </x:rPr>
+          <x:t>Die Tafeln der Formelmappe je Stand als Werte (stand.tabelle.betriebskosten, .kwkg_module, .mehrjahres) und darunter der Zahlungsstrom als Diagramm — ohne Wirtschaftlichkeit bleiben die Zellen leer.</x:t>
+        </x:r>
+      </x:text>
+    </x:comment>
+    <x:comment ref="A15" authorId="0">
+      <x:text>
+        <x:r>
+          <x:rPr>
+            <x:vertAlign val="baseline"/>
+            <x:sz val="9"/>
+            <x:color rgb="FF000000"/>
+            <x:rFont val="Tahoma"/>
+            <x:family val="2"/>
+          </x:rPr>
+          <x:t>Die Betriebskosten des laufenden Stands nach Kostenart mit Bemessung, Herleitung, Betrag und Summe; nur im Block #je stand. Tabelle je Stand als Zellmarke auf dem Musterblatt: je Kopie die Tabelle ihres Stands.</x:t>
+        </x:r>
+      </x:text>
+    </x:comment>
+    <x:comment ref="A17" authorId="0">
+      <x:text>
+        <x:r>
+          <x:rPr>
+            <x:vertAlign val="baseline"/>
+            <x:sz val="9"/>
+            <x:color rgb="FF000000"/>
+            <x:rFont val="Tahoma"/>
+            <x:family val="2"/>
+          </x:rPr>
+          <x:t>Der KWK-Zuschlag des laufenden Stands je BHKW-Modul (elf oder sechzehn Spalten); nur im Block #je stand. Tabelle je Stand als Zellmarke auf dem Musterblatt: je Kopie die Tabelle ihres Stands.</x:t>
+        </x:r>
+      </x:text>
+    </x:comment>
+    <x:comment ref="A19" authorId="0">
+      <x:text>
+        <x:r>
+          <x:rPr>
+            <x:vertAlign val="baseline"/>
+            <x:sz val="9"/>
+            <x:color rgb="FF000000"/>
+            <x:rFont val="Tahoma"/>
+            <x:family val="2"/>
+          </x:rPr>
+          <x:t>Die Mehrjahresübersicht des laufenden Stands: Jahre als Zeilen, Zahlungspositionen als Spalten; nur im Block #je stand. Tabelle je Stand als Zellmarke auf dem Musterblatt: je Kopie die Tabelle ihres Stands.</x:t>
+        </x:r>
+      </x:text>
+    </x:comment>
+    <x:comment ref="A22" authorId="0">
+      <x:text>
+        <x:r>
+          <x:rPr>
+            <x:vertAlign val="baseline"/>
+            <x:sz val="9"/>
+            <x:color rgb="FF000000"/>
+            <x:rFont val="Tahoma"/>
+            <x:family val="2"/>
+          </x:rPr>
+          <x:t>Excel-Tabelle je Stand (EPOS_stand__tabelle__monatswerte) auf dem Musterblatt: Jede Kopie bekommt eine eigene Excel-Tabelle mit den Monatswerten ihres Stands.</x:t>
+        </x:r>
+      </x:text>
+    </x:comment>
+    <x:comment ref="A26" authorId="0">
+      <x:text>
+        <x:r>
+          <x:rPr>
+            <x:vertAlign val="baseline"/>
+            <x:sz val="9"/>
+            <x:color rgb="FF000000"/>
+            <x:rFont val="Tahoma"/>
+            <x:family val="2"/>
+          </x:rPr>
+          <x:t>Bild je Stand: Wärmeerzeugung im Jahresverlauf (gestapelte Erzeuger, Bedarf als Linie, Tagesmittel) — braucht die Stundenreihen des Laufs. Bildplatzhalter: Hier entsteht ein Excel-Diagramm (zehn Spalten × zwanzig Zeilen) mit den Zahlen des Blattes „Diagrammdaten“. Verschieben oder löschen Sie die Zelle; das fertige Diagramm formatieren Sie in Excel.</x:t>
+        </x:r>
+      </x:text>
+    </x:comment>
+    <x:comment ref="A48" authorId="0">
+      <x:text>
+        <x:r>
+          <x:rPr>
+            <x:vertAlign val="baseline"/>
+            <x:sz val="9"/>
+            <x:color rgb="FF000000"/>
+            <x:rFont val="Tahoma"/>
+            <x:family val="2"/>
+          </x:rPr>
+          <x:t>Bild je Stand: Jahresdauerlinie Wärme (geordnete Bedarfs- und Erzeugerdauerlinien) — braucht die Stundenreihen des Laufs. Bildplatzhalter: Hier entsteht ein Excel-Diagramm (zehn Spalten × zwanzig Zeilen) mit den Zahlen des Blattes „Diagrammdaten“. Verschieben oder löschen Sie die Zelle; das fertige Diagramm formatieren Sie in Excel.</x:t>
+        </x:r>
+      </x:text>
+    </x:comment>
+    <x:comment ref="A70" authorId="0">
+      <x:text>
+        <x:r>
+          <x:rPr>
+            <x:vertAlign val="baseline"/>
+            <x:sz val="9"/>
+            <x:color rgb="FF000000"/>
+            <x:rFont val="Tahoma"/>
+            <x:family val="2"/>
+          </x:rPr>
+          <x:t>Bild je Stand: Strombilanz im Monatsverlauf (Deckung gestapelt, Einspeisung, Bedarf als Linie) — braucht die Stundenreihen des Laufs. Bildplatzhalter: Hier entsteht ein Excel-Diagramm (zehn Spalten × zwanzig Zeilen) mit den Zahlen des Blattes „Diagrammdaten“. Verschieben oder löschen Sie die Zelle; das fertige Diagramm formatieren Sie in Excel.</x:t>
+        </x:r>
+      </x:text>
+    </x:comment>
+    <x:comment ref="A92" authorId="0">
+      <x:text>
+        <x:r>
+          <x:rPr>
+            <x:vertAlign val="baseline"/>
+            <x:sz val="9"/>
+            <x:color rgb="FF000000"/>
+            <x:rFont val="Tahoma"/>
+            <x:family val="2"/>
+          </x:rPr>
+          <x:t>Bild je Stand: Speicherverlauf in drei charakteristischen Wochen — braucht die Stundenreihen des Laufs. Bildplatzhalter: Hier entsteht ein Excel-Diagramm (zehn Spalten × zwanzig Zeilen) mit den Zahlen des Blattes „Diagrammdaten“. Verschieben oder löschen Sie die Zelle; das fertige Diagramm formatieren Sie in Excel.</x:t>
+        </x:r>
+      </x:text>
+    </x:comment>
+    <x:comment ref="A114" authorId="0">
+      <x:text>
+        <x:r>
+          <x:rPr>
+            <x:vertAlign val="baseline"/>
+            <x:sz val="9"/>
+            <x:color rgb="FF000000"/>
+            <x:rFont val="Tahoma"/>
+            <x:family val="2"/>
+          </x:rPr>
+          <x:t>Bild je Stand: Anteile der Erzeuger an der Wärmedeckung (Kuchen; der Rest ist ungedeckt). Bildplatzhalter: Hier entsteht ein Excel-Diagramm (zehn Spalten × zwanzig Zeilen) mit den Zahlen des Blattes „Diagrammdaten“. Verschieben oder löschen Sie die Zelle; das fertige Diagramm formatieren Sie in Excel. Deckung Wärme und Strom als Kreis (stand.bild.deckung_waerme, .deckung_strom): Im erzeugten Bericht stehen die Kreise aller Stände auf dem Blatt „Vergleich“, hier auf der Kopie ihres Stands.</x:t>
+        </x:r>
+      </x:text>
+    </x:comment>
+    <x:comment ref="A136" authorId="0">
+      <x:text>
+        <x:r>
+          <x:rPr>
+            <x:vertAlign val="baseline"/>
+            <x:sz val="9"/>
+            <x:color rgb="FF000000"/>
+            <x:rFont val="Tahoma"/>
+            <x:family val="2"/>
+          </x:rPr>
+          <x:t>Bild je Stand: Anteile an der Stromdeckung (Kuchen; der Rest ist Netzbezug). Bildplatzhalter: Hier entsteht ein Excel-Diagramm (zehn Spalten × zwanzig Zeilen) mit den Zahlen des Blattes „Diagrammdaten“. Verschieben oder löschen Sie die Zelle; das fertige Diagramm formatieren Sie in Excel.</x:t>
+        </x:r>
+      </x:text>
+    </x:comment>
+    <x:comment ref="A158" authorId="0">
+      <x:text>
+        <x:r>
+          <x:rPr>
+            <x:vertAlign val="baseline"/>
+            <x:sz val="9"/>
+            <x:color rgb="FF000000"/>
+            <x:rFont val="Tahoma"/>
+            <x:family val="2"/>
+          </x:rPr>
+          <x:t>Bild je Stand: Zahlungsstrom je Jahr im Szenario „Erwartet“ (gestapelte Jahresbalken, Ersatzjahre markiert). Bildplatzhalter: Hier entsteht ein Excel-Diagramm (zehn Spalten × zwanzig Zeilen) mit den Zahlen des Blattes „Diagrammdaten“. Verschieben oder löschen Sie die Zelle; das fertige Diagramm formatieren Sie in Excel.</x:t>
         </x:r>
       </x:text>
     </x:comment>
@@ -530,63 +1076,7 @@
             <x:rFont val="Tahoma"/>
             <x:family val="2"/>
           </x:rPr>
-          <x:t>Musterblatt: Die Blattmarke blatt.detail auf einem Blatt mit weiteren Zellen — EPOS legt je Stand eine Kopie an, benannt wie das Detailblatt, und füllt ihre Platzhalter stand.* mit den Werten dieses Stands.</x:t>
-        </x:r>
-      </x:text>
-    </x:comment>
-    <x:comment ref="A2" authorId="0">
-      <x:text>
-        <x:r>
-          <x:rPr>
-            <x:vertAlign val="baseline"/>
-            <x:sz val="9"/>
-            <x:color rgb="FF000000"/>
-            <x:rFont val="Tahoma"/>
-            <x:family val="2"/>
-          </x:rPr>
-          <x:t>Werte je Stand (stand.*) stehen nur auf dem Musterblatt; Excel kennt keine Blöcke wie Word.</x:t>
-        </x:r>
-      </x:text>
-    </x:comment>
-    <x:comment ref="A10" authorId="0">
-      <x:text>
-        <x:r>
-          <x:rPr>
-            <x:vertAlign val="baseline"/>
-            <x:sz val="9"/>
-            <x:color rgb="FF000000"/>
-            <x:rFont val="Tahoma"/>
-            <x:family val="2"/>
-          </x:rPr>
-          <x:t>Tabelle je Stand als Zellmarke auf dem Musterblatt: je Kopie die Tabelle ihres Stands.</x:t>
-        </x:r>
-      </x:text>
-    </x:comment>
-    <x:comment ref="A13" authorId="0">
-      <x:text>
-        <x:r>
-          <x:rPr>
-            <x:vertAlign val="baseline"/>
-            <x:sz val="9"/>
-            <x:color rgb="FF000000"/>
-            <x:rFont val="Tahoma"/>
-            <x:family val="2"/>
-          </x:rPr>
-          <x:t>Excel-Tabelle je Stand (EPOS_stand__tabelle__monatswerte) auf dem Musterblatt: Jede Kopie bekommt eine eigene Excel-Tabelle mit den Monatswerten ihres Stands.</x:t>
-        </x:r>
-      </x:text>
-    </x:comment>
-    <x:comment ref="A17" authorId="0">
-      <x:text>
-        <x:r>
-          <x:rPr>
-            <x:vertAlign val="baseline"/>
-            <x:sz val="9"/>
-            <x:color rgb="FF000000"/>
-            <x:rFont val="Tahoma"/>
-            <x:family val="2"/>
-          </x:rPr>
-          <x:t>Diagramm je Stand: Der Bildplatzhalter stand.bild.* auf dem Musterblatt wird auf jeder Kopie das Diagramm ihres Stands.</x:t>
+          <x:t>Blattmarke der Checkliste Anhang E: Die Spalte „Stelle im Bericht“ nennt für diese Mappe Blatt und Zelle — die Stelle eines Platzhalters dieser Vorlage, der den Punkt belegt, sonst die Blocküberschrift im erzeugten Blatt. Sie bleibt eine Blattmarke, weil EPOS diese Stellen erst nach dem Füllen aus der fertigen Mappe bestimmt; die Tabelle tabelle.anhang_e.checkliste nennt die Stellen des Wortberichts.</x:t>
         </x:r>
       </x:text>
     </x:comment>
@@ -610,7 +1100,21 @@
             <x:rFont val="Tahoma"/>
             <x:family val="2"/>
           </x:rPr>
-          <x:t>Blattmarke der Checkliste Anhang E: Die Spalte „Stelle im Bericht“ nennt für diese Mappe Blatt und Zelle — die Stelle eines Platzhalters dieser Vorlage, der den Punkt belegt, sonst die Blocküberschrift im erzeugten Blatt.</x:t>
+          <x:t>Excel-Tabelle mit dem Namen EPOS_tabelle__wirtschaft__szenarien: EPOS füllt sie Zeile für Zeile, sie wächst oder schrumpft. Das Säulendiagramm rechts zeigt auf ihre Datenzeilen — EPOS zieht seine Bezüge mit und trägt die neuen Werte ein.</x:t>
+        </x:r>
+      </x:text>
+    </x:comment>
+    <x:comment ref="A29" authorId="0">
+      <x:text>
+        <x:r>
+          <x:rPr>
+            <x:vertAlign val="baseline"/>
+            <x:sz val="9"/>
+            <x:color rgb="FF000000"/>
+            <x:rFont val="Tahoma"/>
+            <x:family val="2"/>
+          </x:rPr>
+          <x:t>Die Namen EPOS.reihe.monate und EPOS.reihe.waermebedarf.monate zeigen hier auf zwölf Zellen; das Liniendiagramm rechts nutzt die Namen. Beim Füllen setzt EPOS die Namen auf die Monatssummen des Stammprojekts im Blatt „Diagrammdaten“.</x:t>
         </x:r>
       </x:text>
     </x:comment>
@@ -735,43 +1239,211 @@
     <x:t>{{bericht.warnungen}}</x:t>
   </x:si>
   <x:si>
-    <x:t>{{blatt.uebersicht}}</x:t>
-  </x:si>
-  <x:si>
-    <x:t>{{blatt.vergleich}}</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Auswertung</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Tabelle der Stände: Rolle, Bezeichner, Projektname, Simulation vom, Hinweis und Stromspeicher. · tabelle.varianten</x:t>
+    <x:t>EPOS-Plan — Variantenvergleich</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Projekt</x:t>
+  </x:si>
+  <x:si>
+    <x:t>{{projekt.name}}</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Kunde</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Bearbeiter</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Klimaregion</x:t>
+  </x:si>
+  <x:si>
+    <x:t>{{projekt.klimaregion}}</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Berichtsdatum</x:t>
+  </x:si>
+  <x:si>
+    <x:t>{{bericht.datum|datum mit zeit}}</x:t>
   </x:si>
   <x:si>
     <x:t>{{tabelle.varianten}}</x:t>
   </x:si>
   <x:si>
-    <x:t>Tabelle Gewerk × Stand: welche Komponenten jeder Stand führt (✓, ✓ (Anzahl) oder —); Spalten je Stand in Blöcken zu drei Varianten. · tabelle.komponenten.matrix</x:t>
-  </x:si>
-  <x:si>
     <x:t>{{tabelle.komponenten.matrix}}</x:t>
   </x:si>
   <x:si>
-    <x:t>Nur Excel: der Parameterblock der Formelmappe — Kalkulationszins, Betrachtungszeitraum, Preissteigerungen und die Änderungen der Szenarien Erwartet, Günstig und Ungünstig als Anteil, die Namen der Formelmappe und die gepflegten Trägerpreise. · tabelle.wirtschaft.parameter</x:t>
+    <x:t>{{stamm.bild.speichertemperaturen}}</x:t>
+  </x:si>
+  <x:si>
+    <x:t>{{tabelle.vergleich.liste}}</x:t>
+  </x:si>
+  <x:si>
+    <x:t>{{bild.vergleich.balken.energie.brennstoff}}</x:t>
+  </x:si>
+  <x:si>
+    <x:t>{{bild.vergleich.balken.energie.netzbezug}}</x:t>
+  </x:si>
+  <x:si>
+    <x:t>{{bild.vergleich.balken.energie.waermerest}}</x:t>
+  </x:si>
+  <x:si>
+    <x:t>{{bild.vergleich.balken.eff.jaz}}</x:t>
+  </x:si>
+  <x:si>
+    <x:t>{{blatt.wirtschaftlichkeit}}</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Wirtschaftlichkeit in Einzelelementen</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Parameter der Wirtschaftlichkeit</x:t>
   </x:si>
   <x:si>
     <x:t>{{tabelle.wirtschaft.parameter}}</x:t>
   </x:si>
   <x:si>
-    <x:t>Nur Excel: der Kapitalwertverlauf je Jahr — je Szenario und Stand eine Spalte, darunter Nulldurchgang, Restwert und Kapitalwertdifferenz (wie das Blatt „Verlauf“); verbundene Köpfe, ein erzeugter Bereich. · tabelle.wirtschaft.verlauf</x:t>
+    <x:t>Kennzahlen — Erwartet</x:t>
+  </x:si>
+  <x:si>
+    <x:t>{{tabelle.wirtschaft.kennzahlen}}</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Kennzahlen — Günstig</x:t>
+  </x:si>
+  <x:si>
+    <x:t>{{tabelle.wirtschaft.kennzahlen.guenstig}}</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Kennzahlen — Ungünstig</x:t>
+  </x:si>
+  <x:si>
+    <x:t>{{tabelle.wirtschaft.kennzahlen.unguenstig}}</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Bandbreite der Szenarien</x:t>
+  </x:si>
+  <x:si>
+    <x:t>{{tabelle.wirtschaft.szenarien}}</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Vorschlag zur Entscheidung</x:t>
+  </x:si>
+  <x:si>
+    <x:t>{{wirtschaft.vorschlag}}</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Nicht monetarisierbare Wirkungen</x:t>
+  </x:si>
+  <x:si>
+    <x:t>{{tabelle.wirtschaft.nicht_monetaer}}</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Hinweise und Warnungen</x:t>
+  </x:si>
+  <x:si>
+    <x:t>{{wirtschaft.hinweise}}</x:t>
+  </x:si>
+  <x:si>
+    <x:t>{{wirtschaft.warnungen}}</x:t>
+  </x:si>
+  <x:si>
+    <x:t>{{bild.wirtschaft.kapitalwert_szenarien}}</x:t>
+  </x:si>
+  <x:si>
+    <x:t>{{bild.wirtschaft.barwerte_kumuliert}}</x:t>
+  </x:si>
+  <x:si>
+    <x:t>{{bild.wirtschaft.bruecke}}</x:t>
+  </x:si>
+  <x:si>
+    <x:t>{{bild.wirtschaft.spanne}}</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Kumulierter Barwert der Differenz zur Referenz je Jahr [€] — ohne Restwert</x:t>
   </x:si>
   <x:si>
     <x:t>{{tabelle.wirtschaft.verlauf}}</x:t>
   </x:si>
   <x:si>
-    <x:t>Bild: Spanne der Kapitalwertdifferenz je Version über die drei Szenarien. · bild.wirtschaft.spanne</x:t>
-  </x:si>
-  <x:si>
-    <x:t>{{bild.wirtschaft.spanne}}</x:t>
+    <x:t>{{blatt.detail}}</x:t>
+  </x:si>
+  <x:si>
+    <x:t>{{stand.rolle}} — {{stand.projektname}}</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Simulationsstand</x:t>
+  </x:si>
+  <x:si>
+    <x:t>{{stand.simulationsstand}}</x:t>
+  </x:si>
+  <x:si>
+    <x:t>{{stand.fehler}}</x:t>
+  </x:si>
+  <x:si>
+    <x:t>{{stand.tabelle.kennzahlen.liste}}</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Erzeuger — Einzelauflistung (Module)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>{{stand.tabelle.erzeuger}}</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Brennstoffmengen</x:t>
+  </x:si>
+  <x:si>
+    <x:t>{{stand.tabelle.brennstoffmengen}}</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Wirtschaftlichkeit dieses Stands</x:t>
+  </x:si>
+  <x:si>
+    <x:t>{{stand.tabelle.betriebskosten}}</x:t>
+  </x:si>
+  <x:si>
+    <x:t>{{stand.tabelle.kwkg_module}}</x:t>
+  </x:si>
+  <x:si>
+    <x:t>{{stand.tabelle.mehrjahres}}</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Monatswerte [MWh] (aus dem Simulationslauf dieses Berichts)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Monat</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Wert</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Musterzeile</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Diagramme</x:t>
+  </x:si>
+  <x:si>
+    <x:t>{{stand.bild.waerme_jahresverlauf}}</x:t>
+  </x:si>
+  <x:si>
+    <x:t>{{stand.bild.waerme_dauerlinie}}</x:t>
+  </x:si>
+  <x:si>
+    <x:t>{{stand.bild.strombilanz_monate}}</x:t>
+  </x:si>
+  <x:si>
+    <x:t>{{stand.bild.speicherverlauf}}</x:t>
+  </x:si>
+  <x:si>
+    <x:t>{{stand.bild.deckung_waerme}}</x:t>
+  </x:si>
+  <x:si>
+    <x:t>{{stand.bild.deckung_strom}}</x:t>
+  </x:si>
+  <x:si>
+    <x:t>{{stand.bild.zahlungsstrom}}</x:t>
+  </x:si>
+  <x:si>
+    <x:t>{{blatt.checkliste}}</x:t>
   </x:si>
   <x:si>
     <x:t>Version</x:t>
@@ -795,9 +1467,6 @@
     <x:t>Einstufung</x:t>
   </x:si>
   <x:si>
-    <x:t>Musterzeile</x:t>
-  </x:si>
-  <x:si>
     <x:t>Jan</x:t>
   </x:si>
   <x:si>
@@ -832,60 +1501,6 @@
   </x:si>
   <x:si>
     <x:t>Dez</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Monat</x:t>
-  </x:si>
-  <x:si>
-    <x:t>{{blatt.wirtschaftlichkeit}}</x:t>
-  </x:si>
-  <x:si>
-    <x:t>{{blatt.verlauf}}</x:t>
-  </x:si>
-  <x:si>
-    <x:t>{{blatt.detail}}</x:t>
-  </x:si>
-  <x:si>
-    <x:t>{{stand.anzeige}}</x:t>
-  </x:si>
-  <x:si>
-    <x:t>{{stand.rolle}}</x:t>
-  </x:si>
-  <x:si>
-    <x:t>{{stand.simulationsstand}}</x:t>
-  </x:si>
-  <x:si>
-    <x:t>{{stand.kennzahl.energie.waermebedarf}}</x:t>
-  </x:si>
-  <x:si>
-    <x:t>{{stand.kennzahl.eff.jaz|stellen 2}}</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Kapitalwertdifferenz</x:t>
-  </x:si>
-  <x:si>
-    <x:t>{{stand.wirtschaft.kapitalwert_diff|mit grund}}</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Die Kernkennzahlen des laufenden Stands als Beschriftung · Wert; nur im Block #je stand. · stand.tabelle.kennzahlen</x:t>
-  </x:si>
-  <x:si>
-    <x:t>{{stand.tabelle.kennzahlen}}</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Nur Excel: die Monatswerte des Stands in MWh aus dem Simulationslauf dieses Berichts — Wärme, Strom, Einspeisung und Netzbezug je Monat; auch als Excel-Tabelle EPOS_stand__tabelle__monatswerte auf dem Musterblatt. · stand.tabelle.monatswerte</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Wert</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Bild je Stand: Strombilanz im Monatsverlauf (Deckung gestapelt, Einspeisung, Bedarf als Linie) — braucht die Stundenreihen des Laufs. · stand.bild.strombilanz_monate</x:t>
-  </x:si>
-  <x:si>
-    <x:t>{{stand.bild.strombilanz_monate}}</x:t>
-  </x:si>
-  <x:si>
-    <x:t>{{blatt.checkliste}}</x:t>
   </x:si>
   <x:si>
     <x:t>{{blatt.diagrammdaten}}</x:t>
@@ -901,7 +1516,7 @@
     <x:numFmt numFmtId="165" formatCode="0.00"/>
     <x:numFmt numFmtId="166" formatCode="#,##0"/>
   </x:numFmts>
-  <x:fonts count="7">
+  <x:fonts count="8">
     <x:font>
       <x:vertAlign val="baseline"/>
       <x:sz val="11"/>
@@ -948,10 +1563,17 @@
       <x:family val="2"/>
     </x:font>
     <x:font>
-      <x:i/>
+      <x:b/>
+      <x:vertAlign val="baseline"/>
+      <x:sz val="13"/>
+      <x:color rgb="FF000000"/>
+      <x:name val="Calibri"/>
+      <x:family val="2"/>
+    </x:font>
+    <x:font>
       <x:vertAlign val="baseline"/>
       <x:sz val="11"/>
-      <x:color rgb="FF7F7F7F"/>
+      <x:color rgb="FFC00000"/>
       <x:name val="Calibri"/>
       <x:family val="2"/>
     </x:font>
@@ -988,7 +1610,7 @@
       </x:diagonal>
     </x:border>
   </x:borders>
-  <x:cellStyleXfs count="11">
+  <x:cellStyleXfs count="12">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
       <x:protection locked="1" hidden="0"/>
     </x:xf>
@@ -1022,8 +1644,11 @@
     <x:xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
       <x:protection locked="1" hidden="0"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
   </x:cellStyleXfs>
-  <x:cellXfs count="12">
+  <x:cellXfs count="13">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
       <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <x:protection locked="1" hidden="0"/>
@@ -1069,6 +1694,10 @@
       <x:protection locked="1" hidden="0"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
+      <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
       <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <x:protection locked="1" hidden="0"/>
     </x:xf>
@@ -1480,7 +2109,7 @@
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rf6a242f4307345ee"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rbbaec054b9ff4951"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1510,7 +2139,7 @@
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R89853625c8f646de"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R332638dc0a0d46d4"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1520,7 +2149,18 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="EPOS_tabelle__wirtschaft__szenarien" displayName="EPOS_tabelle__wirtschaft__szenarien" ref="A1:G2" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="EPOS_stand__tabelle__monatswerte" displayName="EPOS_stand__tabelle__monatswerte" ref="A22:B23" totalsRowShown="0">
+  <x:autoFilter ref="A22:B23"/>
+  <x:tableColumns count="2">
+    <x:tableColumn id="1" name="Monat"/>
+    <x:tableColumn id="2" name="Wert"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="EPOS_tabelle__wirtschaft__szenarien" displayName="EPOS_tabelle__wirtschaft__szenarien" ref="A1:G2" totalsRowShown="0">
   <x:autoFilter ref="A1:G2"/>
   <x:tableColumns count="7">
     <x:tableColumn id="1" name="Version"/>
@@ -1530,17 +2170,6 @@
     <x:tableColumn id="5" name="Spanne"/>
     <x:tableColumn id="6" name="Amortisation"/>
     <x:tableColumn id="7" name="Einstufung"/>
-  </x:tableColumns>
-  <x:tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</x:table>
-</file>
-
-<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="EPOS_stand__tabelle__monatswerte" displayName="EPOS_stand__tabelle__monatswerte" ref="A13:B14" totalsRowShown="0">
-  <x:autoFilter ref="A13:B14"/>
-  <x:tableColumns count="2">
-    <x:tableColumn id="1" name="Monat"/>
-    <x:tableColumn id="2" name="Wert"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -2040,7 +2669,7 @@
   <x:sheetData>
     <x:row r="1" spans="1:7">
       <x:c r="A1" s="0" t="s">
-        <x:v>89</x:v>
+        <x:v>126</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2058,15 +2687,74 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:G1"/>
+  <x:dimension ref="A1:E13"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="7" width="9.140625" style="0" customWidth="1"/>
+    <x:col min="1" max="1" width="22.710625" style="0" customWidth="1"/>
+    <x:col min="2" max="2" width="30.710625" style="0" customWidth="1"/>
+    <x:col min="3" max="3" width="26.710625" style="0" customWidth="1"/>
+    <x:col min="4" max="4" width="18.710625" style="0" customWidth="1"/>
+    <x:col min="5" max="5" width="30.710625" style="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1" spans="1:7">
-      <x:c r="A1" s="0" t="s">
+    <x:row r="1" spans="1:5">
+      <x:c r="A1" s="10" t="s">
         <x:v>38</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" spans="1:5">
+      <x:c r="A3" s="3" t="s">
+        <x:v>39</x:v>
+      </x:c>
+      <x:c r="B3" s="0" t="s">
+        <x:v>40</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" spans="1:5">
+      <x:c r="A4" s="3" t="s">
+        <x:v>41</x:v>
+      </x:c>
+      <x:c r="B4" s="0" t="s">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" spans="1:5">
+      <x:c r="A5" s="3" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="B5" s="0" t="s">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" spans="1:5">
+      <x:c r="A6" s="3" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="B6" s="0" t="s">
+        <x:v>44</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" spans="1:5">
+      <x:c r="A7" s="3" t="s">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="B7" s="0" t="s">
+        <x:v>46</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" spans="1:5">
+      <x:c r="A9" s="0" t="s">
+        <x:v>47</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" spans="1:5">
+      <x:c r="A11" s="0" t="s">
+        <x:v>48</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" spans="1:5">
+      <x:c r="A13" s="0" t="s">
+        <x:v>49</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2084,15 +2772,38 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:G1"/>
+  <x:dimension ref="A1:J69"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="7" width="9.140625" style="0" customWidth="1"/>
+    <x:col min="1" max="1" width="16.710625" style="0" customWidth="1"/>
+    <x:col min="2" max="2" width="42.710625" style="0" customWidth="1"/>
+    <x:col min="3" max="3" width="12.710625" style="0" customWidth="1"/>
+    <x:col min="4" max="10" width="14.710625" style="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1" spans="1:7">
+    <x:row r="1" spans="1:10">
       <x:c r="A1" s="0" t="s">
-        <x:v>39</x:v>
+        <x:v>50</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" spans="1:10">
+      <x:c r="A3" s="0" t="s">
+        <x:v>51</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" spans="1:10">
+      <x:c r="A25" s="0" t="s">
+        <x:v>52</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="47" spans="1:10">
+      <x:c r="A47" s="0" t="s">
+        <x:v>53</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="69" spans="1:10">
+      <x:c r="A69" s="0" t="s">
+        <x:v>54</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2110,66 +2821,15 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:G16"/>
+  <x:dimension ref="A1:G1"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="30.710625" style="0" customWidth="1"/>
-    <x:col min="2" max="7" width="9.140625" style="0" customWidth="1"/>
+    <x:col min="1" max="7" width="9.140625" style="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" spans="1:7">
-      <x:c r="A1" s="10" t="s">
-        <x:v>40</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="3" spans="1:7">
-      <x:c r="A3" s="11" t="s">
-        <x:v>41</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4" spans="1:7">
-      <x:c r="A4" s="0" t="s">
-        <x:v>42</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6" spans="1:7">
-      <x:c r="A6" s="11" t="s">
-        <x:v>43</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7" spans="1:7">
-      <x:c r="A7" s="0" t="s">
-        <x:v>44</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9" spans="1:7">
-      <x:c r="A9" s="11" t="s">
-        <x:v>45</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10" spans="1:7">
-      <x:c r="A10" s="0" t="s">
-        <x:v>46</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12" spans="1:7">
-      <x:c r="A12" s="11" t="s">
-        <x:v>47</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="13" spans="1:7">
-      <x:c r="A13" s="0" t="s">
-        <x:v>48</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="15" spans="1:7">
-      <x:c r="A15" s="11" t="s">
-        <x:v>49</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="16" spans="1:7">
-      <x:c r="A16" s="0" t="s">
-        <x:v>50</x:v>
+      <x:c r="A1" s="0" t="s">
+        <x:v>55</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2187,152 +2847,121 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:G41"/>
+  <x:dimension ref="A1:G94"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="26.710625" style="0" customWidth="1"/>
+    <x:col min="1" max="1" width="44.710625" style="0" customWidth="1"/>
     <x:col min="2" max="7" width="9.140625" style="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" spans="1:7">
-      <x:c r="A1" s="0" t="s">
-        <x:v>51</x:v>
-      </x:c>
-      <x:c r="B1" s="0" t="s">
-        <x:v>52</x:v>
-      </x:c>
-      <x:c r="C1" s="0" t="s">
-        <x:v>53</x:v>
-      </x:c>
-      <x:c r="D1" s="0" t="s">
-        <x:v>54</x:v>
-      </x:c>
-      <x:c r="E1" s="0" t="s">
-        <x:v>55</x:v>
-      </x:c>
-      <x:c r="F1" s="0" t="s">
+      <x:c r="A1" s="10" t="s">
         <x:v>56</x:v>
       </x:c>
-      <x:c r="G1" s="0" t="s">
+    </x:row>
+    <x:row r="3" spans="1:7">
+      <x:c r="A3" s="3" t="s">
         <x:v>57</x:v>
       </x:c>
     </x:row>
-    <x:row r="2" spans="1:7">
-      <x:c r="A2" s="0" t="s">
+    <x:row r="4" spans="1:7">
+      <x:c r="A4" s="0" t="s">
         <x:v>58</x:v>
       </x:c>
-      <x:c r="B2" s="0">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="C2" s="0">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="D2" s="0">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E2" s="0">
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="29" spans="1:7">
-      <x:c r="A29" s="0" t="s">
+    </x:row>
+    <x:row r="6" spans="1:7">
+      <x:c r="A6" s="3" t="s">
+        <x:v>59</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" spans="1:7">
+      <x:c r="A7" s="0" t="s">
+        <x:v>60</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" spans="1:7">
+      <x:c r="A9" s="3" t="s">
+        <x:v>61</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" spans="1:7">
+      <x:c r="A10" s="0" t="s">
+        <x:v>62</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" spans="1:7">
+      <x:c r="A12" s="3" t="s">
+        <x:v>63</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" spans="1:7">
+      <x:c r="A13" s="0" t="s">
+        <x:v>64</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" spans="1:7">
+      <x:c r="A15" s="3" t="s">
+        <x:v>65</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" spans="1:7">
+      <x:c r="A16" s="0" t="s">
+        <x:v>66</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" spans="1:7">
+      <x:c r="A18" s="3" t="s">
+        <x:v>67</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" spans="1:7">
+      <x:c r="A19" s="9" t="s">
+        <x:v>68</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" spans="1:7">
+      <x:c r="A21" s="3" t="s">
+        <x:v>69</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" spans="1:7">
+      <x:c r="A22" s="0" t="s">
+        <x:v>70</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" spans="1:7">
+      <x:c r="A24" s="3" t="s">
         <x:v>71</x:v>
       </x:c>
     </x:row>
-    <x:row r="30" spans="1:7">
-      <x:c r="A30" s="0" t="s">
-        <x:v>59</x:v>
-      </x:c>
-      <x:c r="B30" s="0">
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="31" spans="1:7">
-      <x:c r="A31" s="0" t="s">
-        <x:v>60</x:v>
-      </x:c>
-      <x:c r="B31" s="0">
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="32" spans="1:7">
-      <x:c r="A32" s="0" t="s">
-        <x:v>61</x:v>
-      </x:c>
-      <x:c r="B32" s="0">
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="33" spans="1:7">
-      <x:c r="A33" s="0" t="s">
-        <x:v>62</x:v>
-      </x:c>
-      <x:c r="B33" s="0">
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="34" spans="1:7">
-      <x:c r="A34" s="0" t="s">
-        <x:v>63</x:v>
-      </x:c>
-      <x:c r="B34" s="0">
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="35" spans="1:7">
-      <x:c r="A35" s="0" t="s">
-        <x:v>64</x:v>
-      </x:c>
-      <x:c r="B35" s="0">
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="36" spans="1:7">
-      <x:c r="A36" s="0" t="s">
-        <x:v>65</x:v>
-      </x:c>
-      <x:c r="B36" s="0">
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="37" spans="1:7">
-      <x:c r="A37" s="0" t="s">
-        <x:v>66</x:v>
-      </x:c>
-      <x:c r="B37" s="0">
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="38" spans="1:7">
-      <x:c r="A38" s="0" t="s">
-        <x:v>67</x:v>
-      </x:c>
-      <x:c r="B38" s="0">
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="39" spans="1:7">
-      <x:c r="A39" s="0" t="s">
-        <x:v>68</x:v>
-      </x:c>
-      <x:c r="B39" s="0">
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="40" spans="1:7">
-      <x:c r="A40" s="0" t="s">
-        <x:v>69</x:v>
-      </x:c>
-      <x:c r="B40" s="0">
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="41" spans="1:7">
-      <x:c r="A41" s="0" t="s">
-        <x:v>70</x:v>
-      </x:c>
-      <x:c r="B41" s="0">
-        <x:v>0</x:v>
+    <x:row r="25" spans="1:7">
+      <x:c r="A25" s="9" t="s">
+        <x:v>72</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" spans="1:7">
+      <x:c r="A26" s="9" t="s">
+        <x:v>73</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28" spans="1:7">
+      <x:c r="A28" s="0" t="s">
+        <x:v>74</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="50" spans="1:7">
+      <x:c r="A50" s="0" t="s">
+        <x:v>75</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="72" spans="1:7">
+      <x:c r="A72" s="0" t="s">
+        <x:v>76</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="94" spans="1:7">
+      <x:c r="A94" s="0" t="s">
+        <x:v>77</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2340,15 +2969,198 @@
   <x:pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>
   <x:pageSetup paperSize="1" scale="100" pageOrder="downThenOver" orientation="default" blackAndWhite="0" draft="0" cellComments="none" errors="displayed"/>
   <x:headerFooter/>
-  <x:drawing r:id="R8a5606d9478c4e28"/>
   <x:legacyDrawing r:id="rId23"/>
+  <x:tableParts count="0"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x14ac">
+  <x:sheetPr>
+    <x:outlinePr summaryBelow="1" summaryRight="1"/>
+  </x:sheetPr>
+  <x:dimension ref="A1:G3"/>
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="14.710625" style="0" customWidth="1"/>
+    <x:col min="2" max="7" width="9.140625" style="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" spans="1:7">
+      <x:c r="A1" s="10" t="s">
+        <x:v>78</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" spans="1:7">
+      <x:c r="A3" s="0" t="s">
+        <x:v>79</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
+  <x:pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>
+  <x:pageSetup paperSize="1" scale="100" pageOrder="downThenOver" orientation="default" blackAndWhite="0" draft="0" cellComments="none" errors="displayed"/>
+  <x:headerFooter/>
+  <x:legacyDrawing r:id="rId25"/>
+  <x:tableParts count="0"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x14ac">
+  <x:sheetPr>
+    <x:outlinePr summaryBelow="1" summaryRight="1"/>
+  </x:sheetPr>
+  <x:dimension ref="A1:F158"/>
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="40.710625" style="0" customWidth="1"/>
+    <x:col min="2" max="2" width="22.710625" style="0" customWidth="1"/>
+    <x:col min="3" max="6" width="16.710625" style="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" spans="1:6">
+      <x:c r="A1" s="0" t="s">
+        <x:v>80</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" spans="1:6">
+      <x:c r="A2" s="11" t="s">
+        <x:v>81</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" spans="1:6">
+      <x:c r="A3" s="0" t="s">
+        <x:v>82</x:v>
+      </x:c>
+      <x:c r="B3" s="0" t="s">
+        <x:v>83</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" spans="1:6">
+      <x:c r="A4" s="12" t="s">
+        <x:v>84</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" spans="1:6">
+      <x:c r="A6" s="0" t="s">
+        <x:v>85</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" spans="1:6">
+      <x:c r="A8" s="3" t="s">
+        <x:v>86</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" spans="1:6">
+      <x:c r="A9" s="0" t="s">
+        <x:v>87</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" spans="1:6">
+      <x:c r="A11" s="3" t="s">
+        <x:v>88</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" spans="1:6">
+      <x:c r="A12" s="0" t="s">
+        <x:v>89</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" spans="1:6">
+      <x:c r="A14" s="3" t="s">
+        <x:v>90</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" spans="1:6">
+      <x:c r="A15" s="0" t="s">
+        <x:v>91</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" spans="1:6">
+      <x:c r="A17" s="0" t="s">
+        <x:v>92</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" spans="1:6">
+      <x:c r="A19" s="0" t="s">
+        <x:v>93</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" spans="1:6">
+      <x:c r="A21" s="3" t="s">
+        <x:v>94</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" spans="1:6">
+      <x:c r="A22" s="0" t="s">
+        <x:v>95</x:v>
+      </x:c>
+      <x:c r="B22" s="0" t="s">
+        <x:v>96</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" spans="1:6">
+      <x:c r="A23" s="0" t="s">
+        <x:v>97</x:v>
+      </x:c>
+      <x:c r="B23" s="0">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" spans="1:6">
+      <x:c r="A25" s="3" t="s">
+        <x:v>98</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" spans="1:6">
+      <x:c r="A26" s="0" t="s">
+        <x:v>99</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48" spans="1:6">
+      <x:c r="A48" s="0" t="s">
+        <x:v>100</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="70" spans="1:6">
+      <x:c r="A70" s="0" t="s">
+        <x:v>101</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="92" spans="1:6">
+      <x:c r="A92" s="0" t="s">
+        <x:v>102</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="114" spans="1:6">
+      <x:c r="A114" s="0" t="s">
+        <x:v>103</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="136" spans="1:6">
+      <x:c r="A136" s="0" t="s">
+        <x:v>104</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="158" spans="1:6">
+      <x:c r="A158" s="0" t="s">
+        <x:v>105</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
+  <x:pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>
+  <x:pageSetup paperSize="1" scale="100" pageOrder="downThenOver" orientation="default" blackAndWhite="0" draft="0" cellComments="none" errors="displayed"/>
+  <x:headerFooter/>
+  <x:legacyDrawing r:id="rId27"/>
   <x:tableParts count="1">
-    <x:tablePart r:id="rId24"/>
+    <x:tablePart r:id="rId28"/>
   </x:tableParts>
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x14ac">
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2361,139 +3173,7 @@
   <x:sheetData>
     <x:row r="1" spans="1:7">
       <x:c r="A1" s="0" t="s">
-        <x:v>72</x:v>
-      </x:c>
-    </x:row>
-  </x:sheetData>
-  <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
-  <x:pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>
-  <x:pageSetup paperSize="1" scale="100" pageOrder="downThenOver" orientation="default" blackAndWhite="0" draft="0" cellComments="none" errors="displayed"/>
-  <x:headerFooter/>
-  <x:legacyDrawing r:id="rId26"/>
-  <x:tableParts count="0"/>
-</x:worksheet>
-</file>
-
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x14ac">
-  <x:sheetPr>
-    <x:outlinePr summaryBelow="1" summaryRight="1"/>
-  </x:sheetPr>
-  <x:dimension ref="A1:G1"/>
-  <x:sheetFormatPr defaultRowHeight="15"/>
-  <x:cols>
-    <x:col min="1" max="7" width="9.140625" style="0" customWidth="1"/>
-  </x:cols>
-  <x:sheetData>
-    <x:row r="1" spans="1:7">
-      <x:c r="A1" s="0" t="s">
-        <x:v>73</x:v>
-      </x:c>
-    </x:row>
-  </x:sheetData>
-  <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
-  <x:pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>
-  <x:pageSetup paperSize="1" scale="100" pageOrder="downThenOver" orientation="default" blackAndWhite="0" draft="0" cellComments="none" errors="displayed"/>
-  <x:headerFooter/>
-  <x:legacyDrawing r:id="rId28"/>
-  <x:tableParts count="0"/>
-</x:worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x14ac">
-  <x:sheetPr>
-    <x:outlinePr summaryBelow="1" summaryRight="1"/>
-  </x:sheetPr>
-  <x:dimension ref="A1:F17"/>
-  <x:sheetFormatPr defaultRowHeight="15"/>
-  <x:cols>
-    <x:col min="1" max="1" width="40.710625" style="0" customWidth="1"/>
-    <x:col min="2" max="2" width="22.710625" style="0" customWidth="1"/>
-    <x:col min="3" max="6" width="9.140625" style="0" customWidth="1"/>
-  </x:cols>
-  <x:sheetData>
-    <x:row r="1" spans="1:6">
-      <x:c r="A1" s="0" t="s">
-        <x:v>74</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="2" spans="1:6">
-      <x:c r="A2" s="10" t="s">
-        <x:v>75</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="3" spans="1:6">
-      <x:c r="A3" s="0" t="s">
-        <x:v>76</x:v>
-      </x:c>
-      <x:c r="B3" s="0" t="s">
-        <x:v>77</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5" spans="1:6">
-      <x:c r="A5" s="0" t="s">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="B5" s="0" t="s">
-        <x:v>78</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6" spans="1:6">
-      <x:c r="A6" s="0" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="B6" s="0" t="s">
-        <x:v>79</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7" spans="1:6">
-      <x:c r="A7" s="0" t="s">
-        <x:v>80</x:v>
-      </x:c>
-      <x:c r="B7" s="0" t="s">
-        <x:v>81</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9" spans="1:6">
-      <x:c r="A9" s="11" t="s">
-        <x:v>82</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10" spans="1:6">
-      <x:c r="A10" s="0" t="s">
-        <x:v>83</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12" spans="1:6">
-      <x:c r="A12" s="11" t="s">
-        <x:v>84</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="13" spans="1:6">
-      <x:c r="A13" s="0" t="s">
-        <x:v>71</x:v>
-      </x:c>
-      <x:c r="B13" s="0" t="s">
-        <x:v>85</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="14" spans="1:6">
-      <x:c r="A14" s="0" t="s">
-        <x:v>58</x:v>
-      </x:c>
-      <x:c r="B14" s="0">
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="16" spans="1:6">
-      <x:c r="A16" s="11" t="s">
-        <x:v>86</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="17" spans="1:6">
-      <x:c r="A17" s="0" t="s">
-        <x:v>87</x:v>
+        <x:v>106</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2502,9 +3182,7 @@
   <x:pageSetup paperSize="1" scale="100" pageOrder="downThenOver" orientation="default" blackAndWhite="0" draft="0" cellComments="none" errors="displayed"/>
   <x:headerFooter/>
   <x:legacyDrawing r:id="rId30"/>
-  <x:tableParts count="1">
-    <x:tablePart r:id="rId31"/>
-  </x:tableParts>
+  <x:tableParts count="0"/>
 </x:worksheet>
 </file>
 
@@ -2513,15 +3191,152 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:G1"/>
+  <x:dimension ref="A1:G41"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="7" width="9.140625" style="0" customWidth="1"/>
+    <x:col min="1" max="1" width="26.710625" style="0" customWidth="1"/>
+    <x:col min="2" max="7" width="9.140625" style="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" spans="1:7">
       <x:c r="A1" s="0" t="s">
-        <x:v>88</x:v>
+        <x:v>107</x:v>
+      </x:c>
+      <x:c r="B1" s="0" t="s">
+        <x:v>108</x:v>
+      </x:c>
+      <x:c r="C1" s="0" t="s">
+        <x:v>109</x:v>
+      </x:c>
+      <x:c r="D1" s="0" t="s">
+        <x:v>110</x:v>
+      </x:c>
+      <x:c r="E1" s="0" t="s">
+        <x:v>111</x:v>
+      </x:c>
+      <x:c r="F1" s="0" t="s">
+        <x:v>112</x:v>
+      </x:c>
+      <x:c r="G1" s="0" t="s">
+        <x:v>113</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" spans="1:7">
+      <x:c r="A2" s="0" t="s">
+        <x:v>97</x:v>
+      </x:c>
+      <x:c r="B2" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C2" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D2" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E2" s="0">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29" spans="1:7">
+      <x:c r="A29" s="0" t="s">
+        <x:v>95</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30" spans="1:7">
+      <x:c r="A30" s="0" t="s">
+        <x:v>114</x:v>
+      </x:c>
+      <x:c r="B30" s="0">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31" spans="1:7">
+      <x:c r="A31" s="0" t="s">
+        <x:v>115</x:v>
+      </x:c>
+      <x:c r="B31" s="0">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32" spans="1:7">
+      <x:c r="A32" s="0" t="s">
+        <x:v>116</x:v>
+      </x:c>
+      <x:c r="B32" s="0">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33" spans="1:7">
+      <x:c r="A33" s="0" t="s">
+        <x:v>117</x:v>
+      </x:c>
+      <x:c r="B33" s="0">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34" spans="1:7">
+      <x:c r="A34" s="0" t="s">
+        <x:v>118</x:v>
+      </x:c>
+      <x:c r="B34" s="0">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35" spans="1:7">
+      <x:c r="A35" s="0" t="s">
+        <x:v>119</x:v>
+      </x:c>
+      <x:c r="B35" s="0">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36" spans="1:7">
+      <x:c r="A36" s="0" t="s">
+        <x:v>120</x:v>
+      </x:c>
+      <x:c r="B36" s="0">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37" spans="1:7">
+      <x:c r="A37" s="0" t="s">
+        <x:v>121</x:v>
+      </x:c>
+      <x:c r="B37" s="0">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38" spans="1:7">
+      <x:c r="A38" s="0" t="s">
+        <x:v>122</x:v>
+      </x:c>
+      <x:c r="B38" s="0">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39" spans="1:7">
+      <x:c r="A39" s="0" t="s">
+        <x:v>123</x:v>
+      </x:c>
+      <x:c r="B39" s="0">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40" spans="1:7">
+      <x:c r="A40" s="0" t="s">
+        <x:v>124</x:v>
+      </x:c>
+      <x:c r="B40" s="0">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="41" spans="1:7">
+      <x:c r="A41" s="0" t="s">
+        <x:v>125</x:v>
+      </x:c>
+      <x:c r="B41" s="0">
+        <x:v>0</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2529,7 +3344,10 @@
   <x:pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>
   <x:pageSetup paperSize="1" scale="100" pageOrder="downThenOver" orientation="default" blackAndWhite="0" draft="0" cellComments="none" errors="displayed"/>
   <x:headerFooter/>
-  <x:legacyDrawing r:id="rId33"/>
-  <x:tableParts count="0"/>
+  <x:drawing r:id="R7820a6731f494dd5"/>
+  <x:legacyDrawing r:id="rId32"/>
+  <x:tableParts count="1">
+    <x:tablePart r:id="rId33"/>
+  </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Vorlagen auf Katalogfassung 10 neu erzeugt
Katalog v10 bringt Word-Schlüssel, KatalogfassungWord steigt auf 10:
Sammellauf `alle` zweimal gezogen, zweiter Lauf byte-gleich.

- Ausführliche Vorlage (de/en): im Block je Stand die zehn
  Ergebnisbilder je unter hat.bild.<name>, die Kennwerte des
  Speicherlaufs unter stand.hat_speicherlauf und die solare Deckung.
- Bausteinvorlage: die neuen Schlüssel als Schnellbausteine, dazu die
  Beispiele der Positionsform (Word-Fassung ≥ 8).
- Beispiel-, Standard-, Kurzbericht- und Excel-Vorlagen: nur die neue
  Katalogfassung; die Standardvorlage bleibt kapitelgleich (die neuen
  Bilder gehören zu keinem Kapitel).
- Tests: Rahmenzahl der ausführlichen Vorlage 26, Fassung der Beispiel-
  und Standardvorlage = KatalogfassungWord, Glossarwache mit den
  Positionsbeispielen.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WuTkTgYBbZGmc25Uq4qwuU
</commit_message>
<xml_diff>
--- a/WindowsFormsApplication1/Allgemein/Bericht/Vorlagen/Berichtsvorlage_Excel_Ausfuehrlich.xlsx
+++ b/WindowsFormsApplication1/Allgemein/Bericht/Vorlagen/Berichtsvorlage_Excel_Ausfuehrlich.xlsx
@@ -2109,7 +2109,7 @@
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rbbaec054b9ff4951"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R6ea57d54b0c8459b"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2139,7 +2139,7 @@
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R332638dc0a0d46d4"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R5c6f848936bc4438"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -3344,7 +3344,7 @@
   <x:pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>
   <x:pageSetup paperSize="1" scale="100" pageOrder="downThenOver" orientation="default" blackAndWhite="0" draft="0" cellComments="none" errors="displayed"/>
   <x:headerFooter/>
-  <x:drawing r:id="R7820a6731f494dd5"/>
+  <x:drawing r:id="R48b98b90949c4f89"/>
   <x:legacyDrawing r:id="rId32"/>
   <x:tableParts count="1">
     <x:tablePart r:id="rId33"/>

</xml_diff>

<commit_message>
P4c (6): Berichtsplatzhalter tabelle.pufferauslegung (Katalog v12)
Vorlagenfeld tabelle.pufferauslegung (Kontext Stamm, Kapitel Projekt,
Fassung 12) samt Schalter hat.tabelle.pufferauslegung und Katalogtext
VF_TABELLE__PUFFERAUSLEGUNG de/en: dieselben Eigenschaftspaare wie der
Baustein (eine Quelle, PufferauslegungPaare), je Auslegung eine
Gruppenzeile. WordKontext.Vorlagenfelder: steht der Platzhalter in der
Vorlage, schreibt der Baustein am Standardort nichts. Katalogfassung
11 -> 12, Messlatte v12, alle mitgelieferten Vorlagen mit
Werkzeuge/Berichtsvorlage (alle) neu gebaut, ausführliche Vorlage mit
der Tafel im Kapitel Projekt.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BPMpCujk3rWKNoAC783jJT
</commit_message>
<xml_diff>
--- a/WindowsFormsApplication1/Allgemein/Bericht/Vorlagen/Berichtsvorlage_Excel_Ausfuehrlich.xlsx
+++ b/WindowsFormsApplication1/Allgemein/Bericht/Vorlagen/Berichtsvorlage_Excel_Ausfuehrlich.xlsx
@@ -2109,7 +2109,7 @@
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R560c14b532c841e1"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rcd23cc43645e48ce"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2139,7 +2139,7 @@
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R6ec25a54650b47d3"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R7be13ccaa255423b"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -3344,7 +3344,7 @@
   <x:pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>
   <x:pageSetup paperSize="1" scale="100" pageOrder="downThenOver" orientation="default" blackAndWhite="0" draft="0" cellComments="none" errors="displayed"/>
   <x:headerFooter/>
-  <x:drawing r:id="R0c5d2e741d6b47d9"/>
+  <x:drawing r:id="R410b2ff340c44afc"/>
   <x:legacyDrawing r:id="rId32"/>
   <x:tableParts count="1">
     <x:tablePart r:id="rId33"/>

</xml_diff>

<commit_message>
KU3-6b: Kennzahlen, Katalog v13, Bericht und Szenario der freien Kühlung
KennzahlenKatalog: kaelte.wp.frei und kaelte.wp.frei_stunden (Gruppe
Kälte, Summe der Wärmepumpen, null ohne Wirkung). Vorlagenfeldkatalog:
Fassungsmenge 13 (FASSUNG_FREIE_KUEHLUNG_WP), KATALOGFASSUNG 12 -> 13,
Messlatte v13, alle zehn mitgelieferten Vorlagen mit Berichtsvorlage
alle neu erzeugt. BausteineProjekt: zwei Zeilen im Wärmepumpenblock nur
mit wirksamer freier Kühlung. SzenarioMengen reicht MWh (skaliert) und
Stunden an Summe und Modul durch.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01V9wpg3mpxG7aK2r3MzJ8GQ
</commit_message>
<xml_diff>
--- a/WindowsFormsApplication1/Allgemein/Bericht/Vorlagen/Berichtsvorlage_Excel_Ausfuehrlich.xlsx
+++ b/WindowsFormsApplication1/Allgemein/Bericht/Vorlagen/Berichtsvorlage_Excel_Ausfuehrlich.xlsx
@@ -2109,7 +2109,7 @@
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R1b9491ae4d804477"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rb1f3e4a176c64430"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2139,7 +2139,7 @@
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R4e76ee9c4d1d4b9e"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R0d4529fa54c94e84"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -3344,7 +3344,7 @@
   <x:pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>
   <x:pageSetup paperSize="1" scale="100" pageOrder="downThenOver" orientation="default" blackAndWhite="0" draft="0" cellComments="none" errors="displayed"/>
   <x:headerFooter/>
-  <x:drawing r:id="R10be8861069c4c9c"/>
+  <x:drawing r:id="R6f7c293af19641ea"/>
   <x:legacyDrawing r:id="rId32"/>
   <x:tableParts count="1">
     <x:tablePart r:id="rId33"/>

</xml_diff>

<commit_message>
VW1b: Kennzahlen, Katalog v14 und Bericht der Vorlaufwahl (E88)
KennzahlenKatalog: wp.vorlauf.darunter_stunden und
wp.vorlauf.darueber_stunden (Gruppe Effizienz, Summe über die Module mit
Kennlinienwahl, sonst null). Vorlagenfeldkatalog: Fassungsmenge 14
(FASSUNG_VORLAUFWAHL_WP), KATALOGFASSUNG 13 -> 14, Messlatte v14, alle
zehn mitgelieferten Vorlagen mit Berichtsvorlage alle neu erzeugt.
BausteineProjekt: im Heizkreisabschnitt je Modul mit belegter
Vorlaufwahl die Stunden je Stützstelle und darunter/darüber (Texte
de/en in BerichtTexte). SzenarioMengen reicht die Stunden unverändert
durch. Test VorlaufwahlBerichtTests (4 Fälle).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01V9wpg3mpxG7aK2r3MzJ8GQ
</commit_message>
<xml_diff>
--- a/WindowsFormsApplication1/Allgemein/Bericht/Vorlagen/Berichtsvorlage_Excel_Ausfuehrlich.xlsx
+++ b/WindowsFormsApplication1/Allgemein/Bericht/Vorlagen/Berichtsvorlage_Excel_Ausfuehrlich.xlsx
@@ -2109,7 +2109,7 @@
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rb1f3e4a176c64430"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R4ede842f77004fc0"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2139,7 +2139,7 @@
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R0d4529fa54c94e84"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R3f908abf56fd438b"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -3344,7 +3344,7 @@
   <x:pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>
   <x:pageSetup paperSize="1" scale="100" pageOrder="downThenOver" orientation="default" blackAndWhite="0" draft="0" cellComments="none" errors="displayed"/>
   <x:headerFooter/>
-  <x:drawing r:id="R6f7c293af19641ea"/>
+  <x:drawing r:id="Ra26623fa1e164ca8"/>
   <x:legacyDrawing r:id="rId32"/>
   <x:tableParts count="1">
     <x:tablePart r:id="rId33"/>

</xml_diff>

<commit_message>
VB‑E4: Platzhalter stand.tabelle.wirtschaft_szenarien, Katalog v15
Neuer Katalogeintrag stand.tabelle.wirtschaft_szenarien (Tabelle je Stand,
Word und Excel, Seit 15) über Berichtstabellen.WirtschaftskennzahlenSzenarien
samt Schalter hat.tabelle.wirtschaft_szenarien und Beschreibung
VF_STAND__TABELLE__WIRTSCHAFT_SZENARIEN de/en (VB‑Q8 a). KATALOGFASSUNG und
damit KatalogfassungWord 14 -> 15, eingefrorene Liste v15. Anhang-E-Tafel
des Vorlagenwegs und Checkliste des Excel-Berichts nennen in
VALERI-Darstellung die Tafel „Kennzahlen je Szenario“ (Einzelfall
unverändert). Berichtsbedarf führt den Schlüssel als Wirtschaftswert.
Mitgelieferte Vorlagen über Berichtsvorlage „alle“ neu erzeugt.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/WindowsFormsApplication1/Allgemein/Bericht/Vorlagen/Berichtsvorlage_Excel_Ausfuehrlich.xlsx
+++ b/WindowsFormsApplication1/Allgemein/Bericht/Vorlagen/Berichtsvorlage_Excel_Ausfuehrlich.xlsx
@@ -2109,7 +2109,7 @@
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rb5a2afe5039c442d"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R791dc27438944fc4"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2139,7 +2139,7 @@
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rdc91685c24fd47ab"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Re6bb19f52d904e04"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -3344,7 +3344,7 @@
   <x:pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>
   <x:pageSetup paperSize="1" scale="100" pageOrder="downThenOver" orientation="default" blackAndWhite="0" draft="0" cellComments="none" errors="displayed"/>
   <x:headerFooter/>
-  <x:drawing r:id="R50d24efc52a54d5d"/>
+  <x:drawing r:id="R4e800962bc054c46"/>
   <x:legacyDrawing r:id="rId32"/>
   <x:tableParts count="1">
     <x:tablePart r:id="rId33"/>

</xml_diff>

<commit_message>
KP3-O3a-2: Vorlagenfelder gebaeude.ergebnis.*, Katalog v16, Kurzbericht
Neunzehn Einzelfelder gebaeude.ergebnis.* (Nachtauskühl- und
Sommerlüftungsstunden, Zustand, Art, Aufheizzeit, manuelle Aufheizzeit,
T_a,B, P_auf, Quelle, Rampentage, Σ, längste Rampe, W2-/W1-Tage,
Kappungsstunden, Φ_HL, Φ_RH, Auslegungsgröße, Hinweise W1-W5) und der
Datenschalter hat.aufheizung, alle Seit 16. Die im Entwurf geplante
Fassung 12 war vergeben (Strom/Kälte); KATALOGFASSUNG und
KatalogfassungWord 15 -> 16, eingefrorene Liste v16 (20 neue Schlüssel).
Kurzbericht de/en mit Aufheizabsatz je Gebäude (E58 F4 (b)) und zehntem
Kommentar; Wachen nachgezogen. Mitgelieferte Vorlagen über
Berichtsvorlage „alle“ neu erzeugt, OpenXmlValidator 0 Fehler.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01H9uGe7RdCJxbSxTUPLM6Ta
</commit_message>
<xml_diff>
--- a/WindowsFormsApplication1/Allgemein/Bericht/Vorlagen/Berichtsvorlage_Excel_Ausfuehrlich.xlsx
+++ b/WindowsFormsApplication1/Allgemein/Bericht/Vorlagen/Berichtsvorlage_Excel_Ausfuehrlich.xlsx
@@ -2109,7 +2109,7 @@
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R791dc27438944fc4"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R9ea8613dfd9846f8"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2139,7 +2139,7 @@
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Re6bb19f52d904e04"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Re048faa907064217"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -3344,7 +3344,7 @@
   <x:pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>
   <x:pageSetup paperSize="1" scale="100" pageOrder="downThenOver" orientation="default" blackAndWhite="0" draft="0" cellComments="none" errors="displayed"/>
   <x:headerFooter/>
-  <x:drawing r:id="R4e800962bc054c46"/>
+  <x:drawing r:id="R683c8ed31ea54fd9"/>
   <x:legacyDrawing r:id="rId32"/>
   <x:tableParts count="1">
     <x:tablePart r:id="rId33"/>

</xml_diff>

<commit_message>
UB-E4-c: Berichtsvorlagen auf Katalogfassung 17 neu gebaut
Sammelbefehl alle: Standard, Beispiel, Kurzbericht, Ausfuehrlich, Bausteine, Excel.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/WindowsFormsApplication1/Allgemein/Bericht/Vorlagen/Berichtsvorlage_Excel_Ausfuehrlich.xlsx
+++ b/WindowsFormsApplication1/Allgemein/Bericht/Vorlagen/Berichtsvorlage_Excel_Ausfuehrlich.xlsx
@@ -2109,7 +2109,7 @@
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R9ea8613dfd9846f8"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R733c50b9a88643b4"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2139,7 +2139,7 @@
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Re048faa907064217"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Ra3baf9aca5cb431a"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -3344,7 +3344,7 @@
   <x:pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>
   <x:pageSetup paperSize="1" scale="100" pageOrder="downThenOver" orientation="default" blackAndWhite="0" draft="0" cellComments="none" errors="displayed"/>
   <x:headerFooter/>
-  <x:drawing r:id="R683c8ed31ea54fd9"/>
+  <x:drawing r:id="R759e2cc967034af2"/>
   <x:legacyDrawing r:id="rId32"/>
   <x:tableParts count="1">
     <x:tablePart r:id="rId33"/>

</xml_diff>

<commit_message>
KM3-E3-c: Berichtsvorlagen auf Katalogfassung 18 neu gebaut
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LxWpn8bgrFYtFBXppoeoCL
</commit_message>
<xml_diff>
--- a/WindowsFormsApplication1/Allgemein/Bericht/Vorlagen/Berichtsvorlage_Excel_Ausfuehrlich.xlsx
+++ b/WindowsFormsApplication1/Allgemein/Bericht/Vorlagen/Berichtsvorlage_Excel_Ausfuehrlich.xlsx
@@ -2109,7 +2109,7 @@
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R733c50b9a88643b4"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rda135bfa90f44065"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2139,7 +2139,7 @@
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Ra3baf9aca5cb431a"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rc919a77c26704a54"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -3344,7 +3344,7 @@
   <x:pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>
   <x:pageSetup paperSize="1" scale="100" pageOrder="downThenOver" orientation="default" blackAndWhite="0" draft="0" cellComments="none" errors="displayed"/>
   <x:headerFooter/>
-  <x:drawing r:id="R759e2cc967034af2"/>
+  <x:drawing r:id="R0fc1b4be3bc9426d"/>
   <x:legacyDrawing r:id="rId32"/>
   <x:tableParts count="1">
     <x:tablePart r:id="rId33"/>

</xml_diff>

<commit_message>
K-F2: Rechenproben, Datenbanktest, Messlatte v19, Vorlagen auf v19
RueckkuehlwerkRechenwegTests (ohne Datenbank, je Bauart), K-F1-Proben
auf die Befeuchtung nachgezogen, Gleichwertigkeitsprobe ohne die
Ergebnisspalten des Rueckkuehlwerks, Datenbanktest Kuehlturm an einer
Kopie von 1055. Kennzahlbeschriftung mit (sensibel); Vorgaben samt
Quelle in Entwurf 5.3; Berichtsvorlagen mit dem Werkzeug neu gebaut.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PMW1pznKM9W2VBEzRBXXAt
</commit_message>
<xml_diff>
--- a/WindowsFormsApplication1/Allgemein/Bericht/Vorlagen/Berichtsvorlage_Excel_Ausfuehrlich.xlsx
+++ b/WindowsFormsApplication1/Allgemein/Bericht/Vorlagen/Berichtsvorlage_Excel_Ausfuehrlich.xlsx
@@ -2109,7 +2109,7 @@
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rda135bfa90f44065"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rab20b13cc9d8487a"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2139,7 +2139,7 @@
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rc919a77c26704a54"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rcc8e899f3f88489a"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -3344,7 +3344,7 @@
   <x:pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>
   <x:pageSetup paperSize="1" scale="100" pageOrder="downThenOver" orientation="default" blackAndWhite="0" draft="0" cellComments="none" errors="displayed"/>
   <x:headerFooter/>
-  <x:drawing r:id="R0fc1b4be3bc9426d"/>
+  <x:drawing r:id="R3f8d78558e554cc5"/>
   <x:legacyDrawing r:id="rId32"/>
   <x:tableParts count="1">
     <x:tablePart r:id="rId33"/>

</xml_diff>

<commit_message>
AH-V6: Kurzbericht mit Vorheizsatz, Vorlagen auf Fassung 19, Protokoll
Kurzbericht je Sprache: Absatz 7b {{#wenn hat.vorheizen}} je Gebaeude; alle zehn mitgelieferten Vorlagen mit Werkzeuge/Berichtsvorlage alle neu gebaut (Validator 0 Fehler, wiederholbar); Rumpfwache nachgezogen; Protokoll AH-V6.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01X2CX69qnhXXtc6epxnPUv6
</commit_message>
<xml_diff>
--- a/WindowsFormsApplication1/Allgemein/Bericht/Vorlagen/Berichtsvorlage_Excel_Ausfuehrlich.xlsx
+++ b/WindowsFormsApplication1/Allgemein/Bericht/Vorlagen/Berichtsvorlage_Excel_Ausfuehrlich.xlsx
@@ -2109,7 +2109,7 @@
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rda135bfa90f44065"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R7172aaf8be1d4ca9"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2139,7 +2139,7 @@
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rc919a77c26704a54"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R0726bdda888c4758"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -3344,7 +3344,7 @@
   <x:pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>
   <x:pageSetup paperSize="1" scale="100" pageOrder="downThenOver" orientation="default" blackAndWhite="0" draft="0" cellComments="none" errors="displayed"/>
   <x:headerFooter/>
-  <x:drawing r:id="R0fc1b4be3bc9426d"/>
+  <x:drawing r:id="R09d899c283a34381"/>
   <x:legacyDrawing r:id="rId32"/>
   <x:tableParts count="1">
     <x:tablePart r:id="rId33"/>

</xml_diff>

<commit_message>
K-F2: Messlatte Vorlagenfeldkatalog v20, Berichtsvorlagen auf v20
Messlatte aus dem Testausgabeordner der VorlagenfeldkatalogWacheTests
(v19 plus die 30 Schlüssel kaelte.rk.*). Zehn Vorlagen mit
Werkzeuge/Berichtsvorlage alle neu gebaut, OpenXmlValidator 0 Fehler.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PMW1pznKM9W2VBEzRBXXAt
</commit_message>
<xml_diff>
--- a/WindowsFormsApplication1/Allgemein/Bericht/Vorlagen/Berichtsvorlage_Excel_Ausfuehrlich.xlsx
+++ b/WindowsFormsApplication1/Allgemein/Bericht/Vorlagen/Berichtsvorlage_Excel_Ausfuehrlich.xlsx
@@ -2109,7 +2109,7 @@
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R7172aaf8be1d4ca9"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R40efd187d529493d"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2139,7 +2139,7 @@
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R0726bdda888c4758"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R847b38b9006248db"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -3344,7 +3344,7 @@
   <x:pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>
   <x:pageSetup paperSize="1" scale="100" pageOrder="downThenOver" orientation="default" blackAndWhite="0" draft="0" cellComments="none" errors="displayed"/>
   <x:headerFooter/>
-  <x:drawing r:id="R09d899c283a34381"/>
+  <x:drawing r:id="Ra65599b989ce4e49"/>
   <x:legacyDrawing r:id="rId32"/>
   <x:tableParts count="1">
     <x:tablePart r:id="rId33"/>

</xml_diff>

<commit_message>
SA3b: Kurzbericht 7b mit Halbsatz, Berichtsvorlagen auf Fassung 21
Absatz 7b endet mit {{gebaeude.ergebnis.vorheiz_schnellaufheizung}}
(leer ohne Wirkung), Kommentar 9 nennt das Feld; Werkzeuge/
Berichtsvorlage alle: zehn Vorlagen auf v21, Validator 0 Fehler,
wiederholbar. Rumpf des Kurzberichts in der Dateiwache nachgezogen.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01X2CX69qnhXXtc6epxnPUv6
</commit_message>
<xml_diff>
--- a/WindowsFormsApplication1/Allgemein/Bericht/Vorlagen/Berichtsvorlage_Excel_Ausfuehrlich.xlsx
+++ b/WindowsFormsApplication1/Allgemein/Bericht/Vorlagen/Berichtsvorlage_Excel_Ausfuehrlich.xlsx
@@ -2109,7 +2109,7 @@
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R40efd187d529493d"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R6058296677c54288"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2139,7 +2139,7 @@
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R847b38b9006248db"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R576c26df671f4575"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -3344,7 +3344,7 @@
   <x:pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>
   <x:pageSetup paperSize="1" scale="100" pageOrder="downThenOver" orientation="default" blackAndWhite="0" draft="0" cellComments="none" errors="displayed"/>
   <x:headerFooter/>
-  <x:drawing r:id="Ra65599b989ce4e49"/>
+  <x:drawing r:id="Ra0eb098e54df4860"/>
   <x:legacyDrawing r:id="rId32"/>
   <x:tableParts count="1">
     <x:tablePart r:id="rId33"/>

</xml_diff>

<commit_message>
K-F3: Messlatte Vorlagenfeldkatalog v21, Berichtsvorlagen auf v21
Messlatte aus dem Testausgabeordner der VorlagenfeldkatalogWacheTests
(v20 plus die 30 Schluessel kaelte.rk.teilfrei*). Zehn Vorlagen mit
Werkzeuge/Berichtsvorlage alle neu gebaut, OpenXmlValidator 0 Fehler.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PMW1pznKM9W2VBEzRBXXAt
</commit_message>
<xml_diff>
--- a/WindowsFormsApplication1/Allgemein/Bericht/Vorlagen/Berichtsvorlage_Excel_Ausfuehrlich.xlsx
+++ b/WindowsFormsApplication1/Allgemein/Bericht/Vorlagen/Berichtsvorlage_Excel_Ausfuehrlich.xlsx
@@ -2109,7 +2109,7 @@
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R40efd187d529493d"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Ra732fc616a894805"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2139,7 +2139,7 @@
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R847b38b9006248db"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R671ea6ae91d14bc9"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -3344,7 +3344,7 @@
   <x:pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>
   <x:pageSetup paperSize="1" scale="100" pageOrder="downThenOver" orientation="default" blackAndWhite="0" draft="0" cellComments="none" errors="displayed"/>
   <x:headerFooter/>
-  <x:drawing r:id="Ra65599b989ce4e49"/>
+  <x:drawing r:id="R380d1cf50e5f43d4"/>
   <x:legacyDrawing r:id="rId32"/>
   <x:tableParts count="1">
     <x:tablePart r:id="rId33"/>

</xml_diff>

<commit_message>
K6d: Berichtsvorlagen auf Katalogfassung 23 neu gebaut
Zehn Vorlagen mit Werkzeuge/Berichtsvorlage alle neu erzeugt
(Stilvorlage unveraendert), OpenXmlValidator Office 2007-2021 je
0 Fehler; zweiter Lauf byte-gleich. Bausteinvorlagen de/en mit den
neuen Schnellbausteinen der sechs Kaeltekennzahlen.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UNeGChCYZu2EpgFx4P3q1q
</commit_message>
<xml_diff>
--- a/WindowsFormsApplication1/Allgemein/Bericht/Vorlagen/Berichtsvorlage_Excel_Ausfuehrlich.xlsx
+++ b/WindowsFormsApplication1/Allgemein/Bericht/Vorlagen/Berichtsvorlage_Excel_Ausfuehrlich.xlsx
@@ -2109,7 +2109,7 @@
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R8b3a101e7fcc4c3e"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rea3193f4529c4815"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2139,7 +2139,7 @@
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rfd5f5141d01c4f82"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R084dbf35d528482a"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -3344,7 +3344,7 @@
   <x:pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>
   <x:pageSetup paperSize="1" scale="100" pageOrder="downThenOver" orientation="default" blackAndWhite="0" draft="0" cellComments="none" errors="displayed"/>
   <x:headerFooter/>
-  <x:drawing r:id="R92031a2639a14e23"/>
+  <x:drawing r:id="R348543493bb04b36"/>
   <x:legacyDrawing r:id="rId32"/>
   <x:tableParts count="1">
     <x:tablePart r:id="rId33"/>

</xml_diff>

<commit_message>
KB-7c2: Berichtsvorlagen auf Katalogfassung 24 neu gebaut
Werkzeuge/Berichtsvorlage alle: zehn Vorlagen, OpenXmlValidator
0 Fehler, zweiter Lauf byte-gleich. Inhaltlich nur EPOS.Katalogfassung
= 24 und die Schnellbausteine der Bausteinvorlagen (+ wasser_kosten).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LxWpn8bgrFYtFBXppoeoCL
</commit_message>
<xml_diff>
--- a/WindowsFormsApplication1/Allgemein/Bericht/Vorlagen/Berichtsvorlage_Excel_Ausfuehrlich.xlsx
+++ b/WindowsFormsApplication1/Allgemein/Bericht/Vorlagen/Berichtsvorlage_Excel_Ausfuehrlich.xlsx
@@ -2109,7 +2109,7 @@
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rea3193f4529c4815"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rca11dd845f9f4fdc"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2139,7 +2139,7 @@
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R084dbf35d528482a"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Re893480339944ed3"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -3344,7 +3344,7 @@
   <x:pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>
   <x:pageSetup paperSize="1" scale="100" pageOrder="downThenOver" orientation="default" blackAndWhite="0" draft="0" cellComments="none" errors="displayed"/>
   <x:headerFooter/>
-  <x:drawing r:id="R348543493bb04b36"/>
+  <x:drawing r:id="R61f4e178eb844d2e"/>
   <x:legacyDrawing r:id="rId32"/>
   <x:tableParts count="1">
     <x:tablePart r:id="rId33"/>

</xml_diff>

<commit_message>
SK-4: Berichtsvorlagen auf Katalogfassung 25 neu gebaut
Werkzeuge/Berichtsvorlage alle: zehn Vorlagen, OpenXmlValidator 0 Fehler,
zweiter Lauf byte-gleich.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013wUoTAsWXxMzDv3rM3NCzw
</commit_message>
<xml_diff>
--- a/WindowsFormsApplication1/Allgemein/Bericht/Vorlagen/Berichtsvorlage_Excel_Ausfuehrlich.xlsx
+++ b/WindowsFormsApplication1/Allgemein/Bericht/Vorlagen/Berichtsvorlage_Excel_Ausfuehrlich.xlsx
@@ -2109,7 +2109,7 @@
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rca11dd845f9f4fdc"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rf176504979b74474"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2139,7 +2139,7 @@
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Re893480339944ed3"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Re81a601005524985"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -3344,7 +3344,7 @@
   <x:pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>
   <x:pageSetup paperSize="1" scale="100" pageOrder="downThenOver" orientation="default" blackAndWhite="0" draft="0" cellComments="none" errors="displayed"/>
   <x:headerFooter/>
-  <x:drawing r:id="R61f4e178eb844d2e"/>
+  <x:drawing r:id="R72edcb6b652941ab"/>
   <x:legacyDrawing r:id="rId32"/>
   <x:tableParts count="1">
     <x:tablePart r:id="rId33"/>

</xml_diff>

<commit_message>
6b: Kennzahlen Hilfsstrom, CO2 und Stromsteuer, Katalogfassung 26
Vier Kennzahlen: energie.hilfsstrom (MWh/a), em.co2_hilfsstrom (t/a,
Beschriftung nach Emissionsmodus), ko.stromsteuer_hilfsstrom (gesondert
angesetzt) und ko.stromsteuer_hilfsstrom_gesamt (zum Regelsatz), je
€/a; ohne Hilfsstrom null. Die Steuerbeträge setzt die Wirtschaftlich-
keit im Erwartungsfall am Stand (VariantenDaten) und trägt die Kennzahlen
nach. FASSUNG_HILFSSTROM = 26, Messlatte v26 = v25 + 60 Zeilen, Wache
auf 26, mitgelieferte Vorlagen neu gebaut (Werkzeuge/Berichtsvorlage
alle, Validator 0 Fehler). Test HilfsstromKennzahlTests mit Gegenprobe.
Wiki Berichtsvorlagen, Kosten, Emissionen.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LxWpn8bgrFYtFBXppoeoCL
</commit_message>
<xml_diff>
--- a/WindowsFormsApplication1/Allgemein/Bericht/Vorlagen/Berichtsvorlage_Excel_Ausfuehrlich.xlsx
+++ b/WindowsFormsApplication1/Allgemein/Bericht/Vorlagen/Berichtsvorlage_Excel_Ausfuehrlich.xlsx
@@ -2109,7 +2109,7 @@
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rf176504979b74474"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R1d06878e8b264ba1"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2139,7 +2139,7 @@
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Re81a601005524985"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R8c8790021b7c4027"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -3344,7 +3344,7 @@
   <x:pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>
   <x:pageSetup paperSize="1" scale="100" pageOrder="downThenOver" orientation="default" blackAndWhite="0" draft="0" cellComments="none" errors="displayed"/>
   <x:headerFooter/>
-  <x:drawing r:id="R72edcb6b652941ab"/>
+  <x:drawing r:id="R012e1ccd043340c0"/>
   <x:legacyDrawing r:id="rId32"/>
   <x:tableParts count="1">
     <x:tablePart r:id="rId33"/>

</xml_diff>

<commit_message>
EB-2: Berichtsvorlagen auf Katalogfassung 26 neu gebaut
Werkzeuge/Berichtsvorlage alle: zehn Vorlagen, OpenXmlValidator 0 Fehler.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013wUoTAsWXxMzDv3rM3NCzw
</commit_message>
<xml_diff>
--- a/WindowsFormsApplication1/Allgemein/Bericht/Vorlagen/Berichtsvorlage_Excel_Ausfuehrlich.xlsx
+++ b/WindowsFormsApplication1/Allgemein/Bericht/Vorlagen/Berichtsvorlage_Excel_Ausfuehrlich.xlsx
@@ -2109,7 +2109,7 @@
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rf176504979b74474"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R0b67f54991a84c54"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2139,7 +2139,7 @@
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Re81a601005524985"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R5bfcdfa987ae4801"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -3344,7 +3344,7 @@
   <x:pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>
   <x:pageSetup paperSize="1" scale="100" pageOrder="downThenOver" orientation="default" blackAndWhite="0" draft="0" cellComments="none" errors="displayed"/>
   <x:headerFooter/>
-  <x:drawing r:id="R72edcb6b652941ab"/>
+  <x:drawing r:id="Rae17aceefdb0404e"/>
   <x:legacyDrawing r:id="rId32"/>
   <x:tableParts count="1">
     <x:tablePart r:id="rId33"/>

</xml_diff>

<commit_message>
EB-4: Katalogfassung 27 — Messlatte v27, Berichtsvorlagen neu gebaut
Die drei Kennzahlen der Ergebnisreihen tragen Fassung 27 (v26 von origin,
Hilfsstrom, bleibt). Messlatte Vorlagenfeldkatalog_v27.txt aus dem Lauf
der Wache: die origin-Liste v26 plus Kopfzeile und 45 erzeugte Einträge.
Neun Vorlagen mit Werkzeuge/Berichtsvorlage alle neu gebaut, OpenXml-
Validator 0 Fehler.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013wUoTAsWXxMzDv3rM3NCzw
</commit_message>
<xml_diff>
--- a/WindowsFormsApplication1/Allgemein/Bericht/Vorlagen/Berichtsvorlage_Excel_Ausfuehrlich.xlsx
+++ b/WindowsFormsApplication1/Allgemein/Bericht/Vorlagen/Berichtsvorlage_Excel_Ausfuehrlich.xlsx
@@ -2109,7 +2109,7 @@
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R1d06878e8b264ba1"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R0d96084c2ab04205"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2139,7 +2139,7 @@
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R8c8790021b7c4027"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R7121ba467d2b4d1d"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -3344,7 +3344,7 @@
   <x:pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>
   <x:pageSetup paperSize="1" scale="100" pageOrder="downThenOver" orientation="default" blackAndWhite="0" draft="0" cellComments="none" errors="displayed"/>
   <x:headerFooter/>
-  <x:drawing r:id="R012e1ccd043340c0"/>
+  <x:drawing r:id="Re9683ef42d794936"/>
   <x:legacyDrawing r:id="rId32"/>
   <x:tableParts count="1">
     <x:tablePart r:id="rId33"/>

</xml_diff>